<commit_message>
agegado de minuta de reunion
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="218">
   <si>
     <t>Alumnos</t>
   </si>
@@ -646,6 +646,39 @@
   </si>
   <si>
     <t>4A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conti </t>
+  </si>
+  <si>
+    <t>Candela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aguirre </t>
+  </si>
+  <si>
+    <t>Guadalupe</t>
+  </si>
+  <si>
+    <t>Zamira</t>
+  </si>
+  <si>
+    <t>2D</t>
+  </si>
+  <si>
+    <t>Galiano</t>
+  </si>
+  <si>
+    <t>Sanchez</t>
+  </si>
+  <si>
+    <t>Lionel</t>
+  </si>
+  <si>
+    <t>Vasiliev</t>
+  </si>
+  <si>
+    <t>Fausto</t>
   </si>
 </sst>
 </file>
@@ -4550,7 +4583,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O34"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
@@ -4563,7 +4596,7 @@
     <col min="11" max="12" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4609,68 +4642,54 @@
       <c r="O1" s="52">
         <v>46198</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P1" s="52">
+        <v>46254</v>
+      </c>
+      <c r="Q1" s="52">
+        <v>46268</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
+        <v>33</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="P2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" t="s">
-        <v>193</v>
-      </c>
-      <c r="I2" t="s">
-        <v>193</v>
-      </c>
-      <c r="J2">
-        <f>COUNTIF(E2:I2,"P")</f>
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <f>ROUND(J2*10/4,0)</f>
-        <v>5</v>
-      </c>
-      <c r="L2" t="s">
-        <v>193</v>
-      </c>
-      <c r="M2" t="s">
-        <v>193</v>
-      </c>
-      <c r="N2" t="s">
-        <v>193</v>
-      </c>
-      <c r="O2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>193</v>
+      <c r="E3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="H3" t="s">
         <v>193</v>
@@ -4680,11 +4699,11 @@
       </c>
       <c r="J3">
         <f>COUNTIF(E3:I3,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K3">
         <f>ROUND(J3*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L3" t="s">
         <v>193</v>
@@ -4698,25 +4717,28 @@
       <c r="O3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P3" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>22</v>
+        <v>78</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="H4" t="s">
         <v>193</v>
@@ -4726,11 +4748,11 @@
       </c>
       <c r="J4">
         <f>COUNTIF(E4:I4,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <f>ROUND(J4*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L4" t="s">
         <v>193</v>
@@ -4744,36 +4766,45 @@
       <c r="O4" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="53">
-        <v>5</v>
-      </c>
-      <c r="B5" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="C5" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="D5" s="53" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53" t="s">
-        <v>193</v>
-      </c>
-      <c r="G5" s="54" t="s">
-        <v>194</v>
-      </c>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
+      <c r="P4" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" t="s">
+        <v>193</v>
+      </c>
+      <c r="I5" t="s">
+        <v>193</v>
+      </c>
       <c r="J5">
         <f>COUNTIF(E5:I5,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K5">
         <f>ROUND(J5*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L5" t="s">
         <v>193</v>
@@ -4787,30 +4818,32 @@
       <c r="O5" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" s="54" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
-        <v>6</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="G6"/>
-      <c r="H6" t="s">
-        <v>193</v>
-      </c>
-      <c r="I6" t="s">
-        <v>193</v>
+      <c r="P5" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="53">
+        <v>5</v>
+      </c>
+      <c r="B6" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="C6" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D6" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="53"/>
+      <c r="F6" s="53" t="s">
+        <v>193</v>
+      </c>
+      <c r="G6" s="54" t="s">
+        <v>194</v>
       </c>
       <c r="J6">
         <f>COUNTIF(E6:I6,"P")</f>
@@ -4823,7 +4856,7 @@
       <c r="L6" t="s">
         <v>193</v>
       </c>
-      <c r="M6" s="54" t="s">
+      <c r="M6" t="s">
         <v>193</v>
       </c>
       <c r="N6" t="s">
@@ -4832,44 +4865,47 @@
       <c r="O6" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P6" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="H7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I7" t="s">
         <v>193</v>
       </c>
       <c r="J7">
         <f>COUNTIF(E7:I7,"P")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K7">
         <f>ROUND(J7*10/4,0)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L7" t="s">
         <v>193</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" s="54" t="s">
         <v>193</v>
       </c>
       <c r="N7" t="s">
@@ -4878,36 +4914,45 @@
       <c r="O7" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P7" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>53</v>
       </c>
+      <c r="E8" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F8" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I8" t="s">
         <v>193</v>
       </c>
       <c r="J8">
         <f>COUNTIF(E8:I8,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K8">
         <f>ROUND(J8*10/4,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L8" t="s">
         <v>193</v>
@@ -4921,39 +4966,42 @@
       <c r="O8" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P8" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>187</v>
+        <v>90</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>188</v>
+        <v>91</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
+      </c>
+      <c r="H9" t="s">
+        <v>193</v>
+      </c>
+      <c r="I9" t="s">
+        <v>193</v>
       </c>
       <c r="J9">
         <f>COUNTIF(E9:I9,"P")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <f>ROUND(J9*10/4,0)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L9" t="s">
         <v>193</v>
@@ -4962,76 +5010,61 @@
         <v>193</v>
       </c>
       <c r="N9" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="O9" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P9" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>98</v>
+        <v>207</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>99</v>
+        <v>208</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="G10" s="56"/>
-      <c r="H10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J10">
-        <f>COUNTIF(E10:I10,"P")</f>
-        <v>1</v>
-      </c>
-      <c r="K10">
-        <f>ROUND(J10*10/4,0)</f>
-        <v>3</v>
-      </c>
-      <c r="L10" t="s">
-        <v>193</v>
-      </c>
-      <c r="M10" t="s">
-        <v>193</v>
-      </c>
-      <c r="N10" t="s">
-        <v>193</v>
-      </c>
-      <c r="O10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+        <v>206</v>
+      </c>
+      <c r="F10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="P10" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>104</v>
+        <v>187</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>105</v>
+        <v>188</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F11" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H11" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H11" s="7" t="s">
         <v>22</v>
       </c>
       <c r="I11" s="7" t="s">
@@ -5046,27 +5079,33 @@
         <v>8</v>
       </c>
       <c r="L11" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="M11" t="s">
         <v>193</v>
       </c>
       <c r="N11" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="O11" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P11" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>98</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>38</v>
@@ -5074,19 +5113,20 @@
       <c r="F12" s="7" t="s">
         <v>193</v>
       </c>
+      <c r="G12" s="56"/>
       <c r="H12" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J12">
         <f>COUNTIF(E12:I12,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12">
         <f>ROUND(J12*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L12" t="s">
         <v>193</v>
@@ -5100,39 +5140,48 @@
       <c r="O12" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P12" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="E13" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F13" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="H13" s="7" t="s">
-        <v>193</v>
+      <c r="H13" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="J13">
         <f>COUNTIF(E13:I13,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K13">
         <f>ROUND(J13*10/4,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L13" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="M13" t="s">
         <v>193</v>
@@ -5143,48 +5192,48 @@
       <c r="O13" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P13" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>111</v>
+        <v>34</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="J14">
         <f>COUNTIF(E14:I14,"P")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K14">
         <f>ROUND(J14*10/4,0)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="M14" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="N14" t="s">
         <v>193</v>
@@ -5192,22 +5241,25 @@
       <c r="O14" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P14" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D15" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="57" t="s">
-        <v>22</v>
+        <v>108</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>193</v>
@@ -5220,11 +5272,11 @@
       </c>
       <c r="J15">
         <f>COUNTIF(E15:I15,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15">
         <f>ROUND(J15*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L15" t="s">
         <v>193</v>
@@ -5238,45 +5290,54 @@
       <c r="O15" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P15" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="57" t="s">
+      <c r="E16" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>195</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="J16">
         <f>COUNTIF(E16:I16,"P")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K16">
         <f>ROUND(J16*10/4,0)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L16" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="M16" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="N16" t="s">
         <v>193</v>
@@ -5284,64 +5345,53 @@
       <c r="O16" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P16" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>49</v>
+        <v>204</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>50</v>
+        <v>205</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J17">
-        <f>COUNTIF(E17:I17,"P")</f>
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <f>ROUND(J17*10/4,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L17" t="s">
-        <v>193</v>
-      </c>
-      <c r="M17" t="s">
-        <v>193</v>
-      </c>
-      <c r="N17" t="s">
-        <v>193</v>
-      </c>
+        <v>206</v>
+      </c>
+      <c r="F17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
       <c r="O17" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="P17" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="D18" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="57" t="s">
         <v>22</v>
       </c>
       <c r="F18" s="7" t="s">
@@ -5373,19 +5423,28 @@
       <c r="O18" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P18" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>189</v>
+        <v>40</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D19" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="57" t="s">
         <v>38</v>
+      </c>
+      <c r="E19" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>193</v>
@@ -5398,11 +5457,11 @@
       </c>
       <c r="J19">
         <f>COUNTIF(E19:I19,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19">
         <f>ROUND(J19*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L19" t="s">
         <v>193</v>
@@ -5416,22 +5475,25 @@
       <c r="O19" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P19" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>193</v>
@@ -5444,11 +5506,11 @@
       </c>
       <c r="J20">
         <f>COUNTIF(E20:I20,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20">
         <f>ROUND(J20*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L20" t="s">
         <v>193</v>
@@ -5462,19 +5524,28 @@
       <c r="O20" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P20" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>193</v>
@@ -5487,11 +5558,11 @@
       </c>
       <c r="J21">
         <f>COUNTIF(E21:I21,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21">
         <f>ROUND(J21*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L21" t="s">
         <v>193</v>
@@ -5505,36 +5576,42 @@
       <c r="O21" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P21" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>132</v>
+        <v>189</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>193</v>
       </c>
       <c r="J22">
         <f>COUNTIF(E22:I22,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K22">
         <f>ROUND(J22*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L22" t="s">
         <v>193</v>
@@ -5548,63 +5625,58 @@
       <c r="O22" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P22" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>64</v>
+        <v>203</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J23">
-        <f>COUNTIF(E23:I23,"P")</f>
-        <v>1</v>
-      </c>
-      <c r="K23">
-        <f>ROUND(J23*10/4,0)</f>
-        <v>3</v>
-      </c>
-      <c r="L23" t="s">
-        <v>193</v>
-      </c>
-      <c r="M23" t="s">
-        <v>193</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="F23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
       <c r="N23" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="O23" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="P23" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>136</v>
+        <v>56</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>137</v>
+        <v>57</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="E24" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F24" s="7" t="s">
         <v>193</v>
       </c>
@@ -5616,11 +5688,11 @@
       </c>
       <c r="J24">
         <f>COUNTIF(E24:I24,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24">
         <f>ROUND(J24*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L24" t="s">
         <v>193</v>
@@ -5634,28 +5706,28 @@
       <c r="O24" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P24" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H25" s="7" t="s">
         <v>193</v>
@@ -5665,11 +5737,11 @@
       </c>
       <c r="J25">
         <f>COUNTIF(E25:I25,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K25">
         <f>ROUND(J25*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L25" t="s">
         <v>193</v>
@@ -5683,28 +5755,34 @@
       <c r="O25" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P25" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>14</v>
+        <v>132</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>15</v>
+        <v>191</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H26" t="s">
-        <v>193</v>
-      </c>
-      <c r="I26" t="s">
-        <v>22</v>
+      <c r="F26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>193</v>
       </c>
       <c r="J26">
         <f>COUNTIF(E26:I26,"P")</f>
@@ -5715,85 +5793,131 @@
         <v>5</v>
       </c>
       <c r="L26" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="M26" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="N26" t="s">
         <v>193</v>
       </c>
       <c r="O26" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="P26" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>201</v>
+        <v>64</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>202</v>
+        <v>69</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="F27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
+        <v>53</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J27">
+        <f>COUNTIF(E27:I27,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K27">
+        <f>ROUND(J27*10/4,0)</f>
+        <v>3</v>
+      </c>
       <c r="L27" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="M27" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="N27" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="O27" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="P27" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>198</v>
+        <v>136</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>200</v>
+        <v>137</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="F28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
+        <v>38</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="J28">
+        <f>COUNTIF(E28:I28,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <f>ROUND(J28*10/4,0)</f>
+        <v>0</v>
+      </c>
       <c r="L28" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="M28" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="N28" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="O28" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="P28" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>186</v>
+        <v>139</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>24</v>
+        <v>140</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>17</v>
@@ -5804,86 +5928,107 @@
       <c r="F29" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H29" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" t="s">
-        <v>22</v>
+      <c r="G29" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>193</v>
       </c>
       <c r="J29">
         <f>COUNTIF(E29:I29,"P")</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K29">
         <f>ROUND(J29*10/4,0)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L29" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="M29" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="N29" t="s">
-        <v>22</v>
+        <v>193</v>
       </c>
       <c r="O29" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="P29" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>204</v>
+        <v>14</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>205</v>
+        <v>15</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="F30" s="7"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" t="s">
+        <v>193</v>
+      </c>
+      <c r="I30" t="s">
+        <v>22</v>
+      </c>
+      <c r="J30">
+        <f>COUNTIF(E30:I30,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K30">
+        <f>ROUND(J30*10/4,0)</f>
+        <v>5</v>
+      </c>
+      <c r="L30" t="s">
+        <v>22</v>
+      </c>
+      <c r="M30" t="s">
+        <v>22</v>
+      </c>
+      <c r="N30" t="s">
+        <v>193</v>
+      </c>
       <c r="O30" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P30" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>46</v>
+        <v>201</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>47</v>
+        <v>202</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F31" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J31">
-        <f>COUNTIF(E31:I31,"P")</f>
-        <v>4</v>
-      </c>
-      <c r="K31">
-        <f>ROUND(J31*10/4,0)</f>
-        <v>10</v>
-      </c>
+        <v>199</v>
+      </c>
+      <c r="F31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
       <c r="L31" t="s">
         <v>22</v>
       </c>
@@ -5896,16 +6041,22 @@
       <c r="O31" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P31" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="D32" s="1" t="s">
         <v>199</v>
@@ -5925,71 +6076,279 @@
       <c r="O32" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P32" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>203</v>
+        <v>186</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>80</v>
+        <v>24</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H33" t="s">
+        <v>22</v>
+      </c>
+      <c r="I33" t="s">
+        <v>22</v>
+      </c>
+      <c r="J33">
+        <f>COUNTIF(E33:I33,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K33">
+        <f>ROUND(J33*10/4,0)</f>
+        <v>10</v>
+      </c>
+      <c r="L33" t="s">
+        <v>22</v>
+      </c>
+      <c r="M33" t="s">
+        <v>22</v>
+      </c>
       <c r="N33" t="s">
         <v>22</v>
       </c>
       <c r="O33" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P33" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
+        <v>34</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>211</v>
+      </c>
       <c r="D34" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
+      <c r="Q34" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
+        <v>18</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J35">
+        <f>COUNTIF(E35:I35,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K35">
+        <f>ROUND(J35*10/4,0)</f>
+        <v>10</v>
+      </c>
+      <c r="L35" t="s">
+        <v>22</v>
+      </c>
+      <c r="M35" t="s">
+        <v>22</v>
+      </c>
+      <c r="N35" t="s">
+        <v>22</v>
+      </c>
+      <c r="O35" t="s">
+        <v>22</v>
+      </c>
+      <c r="P35" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>28</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
+      <c r="L36" t="s">
+        <v>22</v>
+      </c>
+      <c r="M36" t="s">
+        <v>22</v>
+      </c>
+      <c r="N36" t="s">
+        <v>22</v>
+      </c>
+      <c r="O36" t="s">
+        <v>22</v>
+      </c>
+      <c r="P36" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
+        <v>35</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F37" s="7"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="7"/>
+      <c r="Q37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
+        <v>36</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="F38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="Q38" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
+        <v>37</v>
+      </c>
+      <c r="D39" s="1"/>
+      <c r="F39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
+        <v>38</v>
+      </c>
+      <c r="D40" s="1"/>
+      <c r="F40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="D41" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E41" s="1">
         <f>COUNTIF(E2:E28,"P")</f>
-        <v>10</v>
-      </c>
-      <c r="F34" s="1">
+        <v>9</v>
+      </c>
+      <c r="F41" s="1">
         <f>COUNTIF(F2:F28,"P")</f>
-        <v>8</v>
-      </c>
-      <c r="H34" s="1">
+        <v>6</v>
+      </c>
+      <c r="H41" s="1">
         <f>COUNTIF(H2:H28,"P")</f>
         <v>7</v>
       </c>
-      <c r="I34" s="57">
+      <c r="I41" s="57">
         <f>COUNTIF(I2:I28,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="L41" s="1">
+        <f>COUNTIF(L2:L31,"P")</f>
         <v>4</v>
       </c>
-      <c r="L34" s="1">
-        <f>COUNTIF(L2:L31,"P")</f>
-        <v>7</v>
-      </c>
-      <c r="M34" s="1">
+      <c r="M41" s="1">
         <f>COUNTIF(M2:M31,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="N41" s="1">
+        <f>COUNTIF(N2:N32,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="O41" s="1">
+        <f>COUNTIF(O2:O33,"P")</f>
         <v>6</v>
       </c>
-      <c r="N34" s="1">
-        <f>COUNTIF(N2:N32,"P")</f>
+      <c r="P41" s="1">
+        <f>COUNTIF(P2:P38,"P")</f>
         <v>6</v>
       </c>
-      <c r="O34" s="1">
-        <f>COUNTIF(O2:O33,"P")</f>
-        <v>8</v>
+      <c r="Q41" s="1">
+        <f>COUNTIF(Q2:Q38,"P")</f>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:O33">
-    <sortCondition ref="O2:O33"/>
-    <sortCondition ref="B2:B33"/>
+  <sortState ref="A2:Q38">
+    <sortCondition ref="Q2:Q38"/>
+    <sortCondition ref="B2:B38"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
subida de patron funcional y minuta
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="222">
   <si>
     <t>Alumnos</t>
   </si>
@@ -597,9 +597,6 @@
     <t>Martinez</t>
   </si>
   <si>
-    <t>fabrizio</t>
-  </si>
-  <si>
     <t>isabella giuliana</t>
   </si>
   <si>
@@ -679,6 +676,21 @@
   </si>
   <si>
     <t>Fausto</t>
+  </si>
+  <si>
+    <t>Ramiro</t>
+  </si>
+  <si>
+    <t>Ibañez</t>
+  </si>
+  <si>
+    <t>Nicole</t>
+  </si>
+  <si>
+    <t>Oyola</t>
+  </si>
+  <si>
+    <t>Fabrizio</t>
   </si>
 </sst>
 </file>
@@ -4583,7 +4595,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:T44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
@@ -4596,7 +4608,7 @@
     <col min="11" max="12" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4625,10 +4637,10 @@
         <v>46163</v>
       </c>
       <c r="J1" t="s">
+        <v>195</v>
+      </c>
+      <c r="K1" t="s">
         <v>196</v>
-      </c>
-      <c r="K1" t="s">
-        <v>197</v>
       </c>
       <c r="L1" s="52">
         <v>46177</v>
@@ -4651,19 +4663,25 @@
       <c r="R1" s="52">
         <v>46275</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S1" s="52">
+        <v>46282</v>
+      </c>
+      <c r="T1" s="52">
+        <v>46289</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>210</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F2" s="7"/>
       <c r="H2" s="7"/>
@@ -4672,353 +4690,347 @@
         <v>22</v>
       </c>
       <c r="Q2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S2" t="s">
+        <v>192</v>
+      </c>
+      <c r="T2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
+        <v>37</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="S3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>193</v>
-      </c>
-      <c r="I3" t="s">
-        <v>193</v>
-      </c>
-      <c r="J3">
-        <f>COUNTIF(E3:I3,"P")</f>
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <f>ROUND(J3*10/4,0)</f>
-        <v>5</v>
-      </c>
-      <c r="L3" t="s">
-        <v>193</v>
-      </c>
-      <c r="M3" t="s">
-        <v>193</v>
-      </c>
-      <c r="N3" t="s">
-        <v>193</v>
-      </c>
-      <c r="O3" t="s">
-        <v>193</v>
-      </c>
-      <c r="P3" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>193</v>
-      </c>
-      <c r="R3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>193</v>
+      <c r="E4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="H4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J4">
         <f>COUNTIF(E4:I4,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4">
         <f>ROUND(J4*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R4" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S4" t="s">
+        <v>192</v>
+      </c>
+      <c r="T4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>22</v>
+        <v>78</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="H5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J5">
         <f>COUNTIF(E5:I5,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <f>ROUND(J5*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R5" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" s="54" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="53">
-        <v>5</v>
-      </c>
-      <c r="B6" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="C6" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="D6" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="S5" t="s">
+        <v>192</v>
+      </c>
+      <c r="T5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="53"/>
-      <c r="F6" s="53" t="s">
-        <v>193</v>
-      </c>
-      <c r="G6" s="54" t="s">
-        <v>194</v>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G6"/>
+      <c r="H6" t="s">
+        <v>192</v>
+      </c>
+      <c r="I6" t="s">
+        <v>22</v>
       </c>
       <c r="J6">
         <f>COUNTIF(E6:I6,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K6">
         <f>ROUND(J6*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L6" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="M6" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="N6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O6" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="P6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q6" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="R6" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="S6" t="s">
+        <v>22</v>
+      </c>
+      <c r="T6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>78</v>
+        <v>38</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J7">
         <f>COUNTIF(E7:I7,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K7">
         <f>ROUND(J7*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L7" t="s">
+        <v>192</v>
+      </c>
+      <c r="M7" t="s">
+        <v>192</v>
+      </c>
+      <c r="N7" t="s">
+        <v>192</v>
+      </c>
+      <c r="O7" t="s">
+        <v>192</v>
+      </c>
+      <c r="P7" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>192</v>
+      </c>
+      <c r="R7" t="s">
+        <v>192</v>
+      </c>
+      <c r="S7" t="s">
+        <v>192</v>
+      </c>
+      <c r="T7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>30</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="L8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M8" t="s">
+        <v>22</v>
+      </c>
+      <c r="N8" t="s">
+        <v>22</v>
+      </c>
+      <c r="O8" t="s">
+        <v>22</v>
+      </c>
+      <c r="P8" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>22</v>
+      </c>
+      <c r="R8" t="s">
+        <v>22</v>
+      </c>
+      <c r="S8" t="s">
+        <v>192</v>
+      </c>
+      <c r="T8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9" s="53">
+        <v>5</v>
+      </c>
+      <c r="B9" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="C9" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D9" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="53"/>
+      <c r="F9" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="G9" s="54" t="s">
         <v>193</v>
       </c>
-      <c r="M7" s="54" t="s">
-        <v>193</v>
-      </c>
-      <c r="N7" t="s">
-        <v>193</v>
-      </c>
-      <c r="O7" t="s">
-        <v>193</v>
-      </c>
-      <c r="P7" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>193</v>
-      </c>
-      <c r="R7" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>7</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H8" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" t="s">
-        <v>193</v>
-      </c>
-      <c r="J8">
-        <f>COUNTIF(E8:I8,"P")</f>
-        <v>3</v>
-      </c>
-      <c r="K8">
-        <f>ROUND(J8*10/4,0)</f>
-        <v>8</v>
-      </c>
-      <c r="L8" t="s">
-        <v>193</v>
-      </c>
-      <c r="M8" t="s">
-        <v>193</v>
-      </c>
-      <c r="N8" t="s">
-        <v>193</v>
-      </c>
-      <c r="O8" t="s">
-        <v>193</v>
-      </c>
-      <c r="P8" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>193</v>
-      </c>
-      <c r="R8" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H9" t="s">
-        <v>193</v>
-      </c>
-      <c r="I9" t="s">
-        <v>193</v>
-      </c>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
       <c r="J9">
         <f>COUNTIF(E9:I9,"P")</f>
         <v>0</v>
@@ -5028,167 +5040,219 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R9" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S9" t="s">
+        <v>192</v>
+      </c>
+      <c r="T9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>187</v>
+        <v>84</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>188</v>
+        <v>85</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>195</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
+      </c>
+      <c r="H10" t="s">
+        <v>192</v>
+      </c>
+      <c r="I10" t="s">
+        <v>192</v>
       </c>
       <c r="J10">
         <f>COUNTIF(E10:I10,"P")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K10">
         <f>ROUND(J10*10/4,0)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>193</v>
-      </c>
-      <c r="M10" t="s">
-        <v>193</v>
+        <v>192</v>
+      </c>
+      <c r="M10" s="54" t="s">
+        <v>192</v>
       </c>
       <c r="N10" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="O10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R10" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S10" t="s">
+        <v>192</v>
+      </c>
+      <c r="T10" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="G11" s="56"/>
-      <c r="H11" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
+      </c>
+      <c r="H11" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" t="s">
+        <v>192</v>
       </c>
       <c r="J11">
         <f>COUNTIF(E11:I11,"P")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K11">
         <f>ROUND(J11*10/4,0)</f>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="L11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R11" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S11" t="s">
+        <v>192</v>
+      </c>
+      <c r="T11" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>213</v>
+        <v>90</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>211</v>
+        <v>91</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="F12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+        <v>53</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H12" t="s">
+        <v>192</v>
+      </c>
+      <c r="I12" t="s">
+        <v>192</v>
+      </c>
+      <c r="J12">
+        <f>COUNTIF(E12:I12,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <f>ROUND(J12*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" t="s">
+        <v>192</v>
+      </c>
+      <c r="M12" t="s">
+        <v>192</v>
+      </c>
+      <c r="N12" t="s">
+        <v>192</v>
+      </c>
+      <c r="O12" t="s">
+        <v>192</v>
+      </c>
+      <c r="P12" t="s">
+        <v>192</v>
+      </c>
       <c r="Q12" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R12" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S12" t="s">
+        <v>192</v>
+      </c>
+      <c r="T12" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>104</v>
+        <v>186</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>105</v>
+        <v>24</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>17</v>
@@ -5197,337 +5261,304 @@
         <v>22</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H13" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" t="s">
         <v>22</v>
       </c>
       <c r="J13">
         <f>COUNTIF(E13:I13,"P")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13">
         <f>ROUND(J13*10/4,0)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L13" t="s">
         <v>22</v>
       </c>
       <c r="M13" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="N13" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="O13" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="P13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q13" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="R13" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="S13" t="s">
+        <v>22</v>
+      </c>
+      <c r="T13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>206</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>35</v>
+        <v>207</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J14">
-        <f>COUNTIF(E14:I14,"P")</f>
-        <v>0</v>
-      </c>
-      <c r="K14">
-        <f>ROUND(J14*10/4,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L14" t="s">
-        <v>193</v>
-      </c>
-      <c r="M14" t="s">
-        <v>193</v>
-      </c>
-      <c r="N14" t="s">
-        <v>193</v>
-      </c>
-      <c r="O14" t="s">
-        <v>193</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="F14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
       <c r="P14" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="Q14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R14" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="S14" t="s">
+        <v>192</v>
+      </c>
+      <c r="T14" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>107</v>
+        <v>187</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>108</v>
+        <v>188</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>194</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="J15">
         <f>COUNTIF(E15:I15,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K15">
         <f>ROUND(J15*10/4,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N15" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="O15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R15" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S15" t="s">
+        <v>192</v>
+      </c>
+      <c r="T15" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>195</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="G16" s="56"/>
       <c r="H16" s="7" t="s">
         <v>22</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="J16">
         <f>COUNTIF(E16:I16,"P")</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K16">
         <f>ROUND(J16*10/4,0)</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L16" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="M16" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="N16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R16" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S16" t="s">
+        <v>192</v>
+      </c>
+      <c r="T16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>113</v>
+        <v>218</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D17" s="57" t="s">
+        <v>219</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="S17" t="s">
+        <v>22</v>
+      </c>
+      <c r="T17" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
+        <v>13</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J17">
-        <f>COUNTIF(E17:I17,"P")</f>
-        <v>1</v>
-      </c>
-      <c r="K17">
-        <f>ROUND(J17*10/4,0)</f>
-        <v>3</v>
-      </c>
-      <c r="L17" t="s">
-        <v>193</v>
-      </c>
-      <c r="M17" t="s">
-        <v>193</v>
-      </c>
-      <c r="N17" t="s">
-        <v>193</v>
-      </c>
-      <c r="O17" t="s">
-        <v>193</v>
-      </c>
-      <c r="P17" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>193</v>
-      </c>
-      <c r="R17" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="1">
-        <v>17</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E18" s="57" t="s">
-        <v>22</v>
-      </c>
       <c r="F18" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J18">
         <f>COUNTIF(E18:I18,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18">
         <f>ROUND(J18*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R18" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S18" t="s">
+        <v>192</v>
+      </c>
+      <c r="T18" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>50</v>
+        <v>108</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J19">
         <f>COUNTIF(E19:I19,"P")</f>
@@ -5538,781 +5569,888 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R19" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S19" t="s">
+        <v>192</v>
+      </c>
+      <c r="T19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>118</v>
+        <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>194</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="J20">
         <f>COUNTIF(E20:I20,"P")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K20">
         <f>ROUND(J20*10/4,0)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L20" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="M20" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="N20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R20" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S20" t="s">
+        <v>192</v>
+      </c>
+      <c r="T20" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>189</v>
+        <v>113</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D21" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D21" s="57" t="s">
         <v>38</v>
       </c>
+      <c r="E21" s="57" t="s">
+        <v>22</v>
+      </c>
       <c r="F21" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J21">
         <f>COUNTIF(E21:I21,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21">
         <f>ROUND(J21*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R21" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S21" t="s">
+        <v>192</v>
+      </c>
+      <c r="T21" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>203</v>
+        <v>40</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
+        <v>41</v>
+      </c>
+      <c r="D22" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H22" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J22">
+        <f>COUNTIF(E22:I22,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K22">
+        <f>ROUND(J22*10/4,0)</f>
+        <v>3</v>
+      </c>
+      <c r="L22" t="s">
+        <v>192</v>
+      </c>
+      <c r="M22" t="s">
+        <v>192</v>
+      </c>
       <c r="N22" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="O22" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="P22" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q22" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R22" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S22" t="s">
+        <v>192</v>
+      </c>
+      <c r="T22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J23">
         <f>COUNTIF(E23:I23,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23">
         <f>ROUND(J23*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R23" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S23" t="s">
+        <v>192</v>
+      </c>
+      <c r="T23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>130</v>
+        <v>118</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J24">
         <f>COUNTIF(E24:I24,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24">
         <f>ROUND(J24*10/4,0)</f>
+        <v>3</v>
+      </c>
+      <c r="L24" t="s">
+        <v>192</v>
+      </c>
+      <c r="M24" t="s">
+        <v>192</v>
+      </c>
+      <c r="N24" t="s">
+        <v>192</v>
+      </c>
+      <c r="O24" t="s">
+        <v>192</v>
+      </c>
+      <c r="P24" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>192</v>
+      </c>
+      <c r="R24" t="s">
+        <v>192</v>
+      </c>
+      <c r="S24" t="s">
+        <v>192</v>
+      </c>
+      <c r="T24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>21</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H25" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J25">
+        <f>COUNTIF(E25:I25,"P")</f>
         <v>0</v>
       </c>
-      <c r="L24" t="s">
-        <v>193</v>
-      </c>
-      <c r="M24" t="s">
-        <v>193</v>
-      </c>
-      <c r="N24" t="s">
-        <v>193</v>
-      </c>
-      <c r="O24" t="s">
-        <v>193</v>
-      </c>
-      <c r="P24" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>193</v>
-      </c>
-      <c r="R24" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>35</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="F25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
+      <c r="K25">
+        <f>ROUND(J25*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L25" t="s">
+        <v>192</v>
+      </c>
+      <c r="M25" t="s">
+        <v>192</v>
+      </c>
+      <c r="N25" t="s">
+        <v>192</v>
+      </c>
+      <c r="O25" t="s">
+        <v>192</v>
+      </c>
+      <c r="P25" t="s">
+        <v>192</v>
+      </c>
       <c r="Q25" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R25" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S25" t="s">
+        <v>192</v>
+      </c>
+      <c r="T25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>132</v>
+        <v>202</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>191</v>
+        <v>80</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J26">
-        <f>COUNTIF(E26:I26,"P")</f>
-        <v>2</v>
-      </c>
-      <c r="K26">
-        <f>ROUND(J26*10/4,0)</f>
-        <v>5</v>
-      </c>
-      <c r="L26" t="s">
-        <v>193</v>
-      </c>
-      <c r="M26" t="s">
-        <v>193</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="F26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
       <c r="N26" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="O26" t="s">
-        <v>193</v>
+        <v>22</v>
       </c>
       <c r="P26" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q26" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R26" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S26" t="s">
+        <v>192</v>
+      </c>
+      <c r="T26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>64</v>
+        <v>220</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>193</v>
-      </c>
-      <c r="J27">
-        <f>COUNTIF(E27:I27,"P")</f>
-        <v>1</v>
-      </c>
-      <c r="K27">
-        <f>ROUND(J27*10/4,0)</f>
-        <v>3</v>
-      </c>
-      <c r="L27" t="s">
-        <v>193</v>
-      </c>
-      <c r="M27" t="s">
-        <v>193</v>
-      </c>
-      <c r="N27" t="s">
-        <v>193</v>
-      </c>
-      <c r="O27" t="s">
-        <v>193</v>
-      </c>
-      <c r="P27" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q27" t="s">
-        <v>193</v>
-      </c>
-      <c r="R27" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+        <v>211</v>
+      </c>
+      <c r="F27" s="7"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="S27" t="s">
+        <v>22</v>
+      </c>
+      <c r="T27" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>136</v>
+        <v>56</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>137</v>
+        <v>57</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="E28" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F28" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J28">
         <f>COUNTIF(E28:I28,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28">
         <f>ROUND(J28*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="M28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="N28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q28" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R28" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S28" t="s">
+        <v>192</v>
+      </c>
+      <c r="T28" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="J29">
         <f>COUNTIF(E29:I29,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K29">
         <f>ROUND(J29*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L29" t="s">
+        <v>192</v>
+      </c>
+      <c r="M29" t="s">
+        <v>192</v>
+      </c>
+      <c r="N29" t="s">
+        <v>192</v>
+      </c>
+      <c r="O29" t="s">
+        <v>192</v>
+      </c>
+      <c r="P29" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>192</v>
+      </c>
+      <c r="R29" t="s">
+        <v>192</v>
+      </c>
+      <c r="S29" t="s">
+        <v>192</v>
+      </c>
+      <c r="T29" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
+        <v>35</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F30" s="7"/>
+      <c r="H30" s="7"/>
+      <c r="I30" s="7"/>
+      <c r="Q30" t="s">
+        <v>22</v>
+      </c>
+      <c r="R30" t="s">
+        <v>192</v>
+      </c>
+      <c r="S30" t="s">
+        <v>192</v>
+      </c>
+      <c r="T30" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
+        <v>24</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H31" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J31">
+        <f>COUNTIF(E31:I31,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K31">
+        <f>ROUND(J31*10/4,0)</f>
         <v>5</v>
       </c>
-      <c r="L29" t="s">
-        <v>193</v>
-      </c>
-      <c r="M29" t="s">
-        <v>193</v>
-      </c>
-      <c r="N29" t="s">
-        <v>193</v>
-      </c>
-      <c r="O29" t="s">
-        <v>193</v>
-      </c>
-      <c r="P29" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>193</v>
-      </c>
-      <c r="R29" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
+      <c r="L31" t="s">
+        <v>192</v>
+      </c>
+      <c r="M31" t="s">
+        <v>192</v>
+      </c>
+      <c r="N31" t="s">
+        <v>192</v>
+      </c>
+      <c r="O31" t="s">
+        <v>192</v>
+      </c>
+      <c r="P31" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>192</v>
+      </c>
+      <c r="R31" t="s">
+        <v>192</v>
+      </c>
+      <c r="S31" t="s">
+        <v>192</v>
+      </c>
+      <c r="T31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
+        <v>25</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H32" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J32">
+        <f>COUNTIF(E32:I32,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K32">
+        <f>ROUND(J32*10/4,0)</f>
         <v>3</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="1" t="s">
+      <c r="L32" t="s">
+        <v>192</v>
+      </c>
+      <c r="M32" t="s">
+        <v>192</v>
+      </c>
+      <c r="N32" t="s">
+        <v>192</v>
+      </c>
+      <c r="O32" t="s">
+        <v>192</v>
+      </c>
+      <c r="P32" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>192</v>
+      </c>
+      <c r="R32" t="s">
+        <v>192</v>
+      </c>
+      <c r="S32" t="s">
+        <v>192</v>
+      </c>
+      <c r="T32" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
+        <v>36</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F33" s="7"/>
+      <c r="H33" s="7"/>
+      <c r="I33" s="7"/>
+      <c r="Q33" t="s">
+        <v>22</v>
+      </c>
+      <c r="R33" t="s">
+        <v>22</v>
+      </c>
+      <c r="S33" t="s">
+        <v>192</v>
+      </c>
+      <c r="T33" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
+        <v>26</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J34">
+        <f>COUNTIF(E34:I34,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K34">
+        <f>ROUND(J34*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L34" t="s">
+        <v>192</v>
+      </c>
+      <c r="M34" t="s">
+        <v>192</v>
+      </c>
+      <c r="N34" t="s">
+        <v>192</v>
+      </c>
+      <c r="O34" t="s">
+        <v>192</v>
+      </c>
+      <c r="P34" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>192</v>
+      </c>
+      <c r="R34" t="s">
+        <v>192</v>
+      </c>
+      <c r="S34" t="s">
+        <v>192</v>
+      </c>
+      <c r="T34" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
+        <v>27</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D35" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H30" t="s">
-        <v>193</v>
-      </c>
-      <c r="I30" t="s">
-        <v>22</v>
-      </c>
-      <c r="J30">
-        <f>COUNTIF(E30:I30,"P")</f>
+      <c r="E35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J35">
+        <f>COUNTIF(E35:I35,"P")</f>
         <v>2</v>
       </c>
-      <c r="K30">
-        <f>ROUND(J30*10/4,0)</f>
+      <c r="K35">
+        <f>ROUND(J35*10/4,0)</f>
         <v>5</v>
       </c>
-      <c r="L30" t="s">
-        <v>22</v>
-      </c>
-      <c r="M30" t="s">
-        <v>22</v>
-      </c>
-      <c r="N30" t="s">
-        <v>193</v>
-      </c>
-      <c r="O30" t="s">
-        <v>22</v>
-      </c>
-      <c r="P30" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>22</v>
-      </c>
-      <c r="R30" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A31" s="1">
-        <v>30</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="D31" s="1" t="s">
+      <c r="L35" t="s">
+        <v>192</v>
+      </c>
+      <c r="M35" t="s">
+        <v>192</v>
+      </c>
+      <c r="N35" t="s">
+        <v>192</v>
+      </c>
+      <c r="O35" t="s">
+        <v>192</v>
+      </c>
+      <c r="P35" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>192</v>
+      </c>
+      <c r="R35" t="s">
+        <v>192</v>
+      </c>
+      <c r="S35" t="s">
+        <v>192</v>
+      </c>
+      <c r="T35" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>29</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="F31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="L31" t="s">
-        <v>22</v>
-      </c>
-      <c r="M31" t="s">
-        <v>22</v>
-      </c>
-      <c r="N31" t="s">
-        <v>22</v>
-      </c>
-      <c r="O31" t="s">
-        <v>22</v>
-      </c>
-      <c r="P31" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q31" t="s">
-        <v>22</v>
-      </c>
-      <c r="R31" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A32" s="1">
-        <v>29</v>
-      </c>
-      <c r="B32" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="F32" s="7"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
-      <c r="L32" t="s">
-        <v>22</v>
-      </c>
-      <c r="M32" t="s">
-        <v>22</v>
-      </c>
-      <c r="N32" t="s">
-        <v>22</v>
-      </c>
-      <c r="O32" t="s">
-        <v>22</v>
-      </c>
-      <c r="P32" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>22</v>
-      </c>
-      <c r="R32" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A33" s="1">
-        <v>9</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H33" t="s">
-        <v>22</v>
-      </c>
-      <c r="I33" t="s">
-        <v>22</v>
-      </c>
-      <c r="J33">
-        <f>COUNTIF(E33:I33,"P")</f>
-        <v>4</v>
-      </c>
-      <c r="K33">
-        <f>ROUND(J33*10/4,0)</f>
-        <v>10</v>
-      </c>
-      <c r="L33" t="s">
-        <v>22</v>
-      </c>
-      <c r="M33" t="s">
-        <v>22</v>
-      </c>
-      <c r="N33" t="s">
-        <v>22</v>
-      </c>
-      <c r="O33" t="s">
-        <v>22</v>
-      </c>
-      <c r="P33" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>22</v>
-      </c>
-      <c r="R33" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34" s="1">
-        <v>32</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="F34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="P34" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>193</v>
-      </c>
-      <c r="R34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A35" s="1">
-        <v>32</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="F35" s="7"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
-      <c r="O35" t="s">
-        <v>22</v>
-      </c>
-      <c r="P35" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q35" t="s">
-        <v>193</v>
-      </c>
-      <c r="R35" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A36" s="1">
-        <v>18</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E36" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F36" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J36">
-        <f>COUNTIF(E36:I36,"P")</f>
-        <v>4</v>
-      </c>
-      <c r="K36">
-        <f>ROUND(J36*10/4,0)</f>
-        <v>10</v>
-      </c>
+      <c r="F36" s="7"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="7"/>
       <c r="L36" t="s">
         <v>22</v>
       </c>
@@ -6334,139 +6472,322 @@
       <c r="R36" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="S36" t="s">
+        <v>192</v>
+      </c>
+      <c r="T36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>188</v>
+        <v>210</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="F37" s="7"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
-      <c r="L37" t="s">
-        <v>22</v>
-      </c>
-      <c r="M37" t="s">
-        <v>22</v>
-      </c>
-      <c r="N37" t="s">
-        <v>22</v>
-      </c>
-      <c r="O37" t="s">
-        <v>22</v>
-      </c>
-      <c r="P37" t="s">
-        <v>22</v>
-      </c>
       <c r="Q37" t="s">
         <v>22</v>
       </c>
       <c r="R37" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S37" t="s">
+        <v>22</v>
+      </c>
+      <c r="T37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>216</v>
+        <v>104</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>217</v>
+        <v>105</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="F38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H38" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J38">
+        <f>COUNTIF(E38:I38,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="K38">
+        <f>ROUND(J38*10/4,0)</f>
+        <v>8</v>
+      </c>
+      <c r="L38" t="s">
+        <v>22</v>
+      </c>
+      <c r="M38" t="s">
+        <v>192</v>
+      </c>
+      <c r="N38" t="s">
+        <v>192</v>
+      </c>
+      <c r="O38" t="s">
+        <v>192</v>
+      </c>
+      <c r="P38" t="s">
+        <v>192</v>
+      </c>
       <c r="Q38" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R38" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="S38" t="s">
+        <v>22</v>
+      </c>
+      <c r="T38" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
-        <v>37</v>
-      </c>
-      <c r="D39" s="1"/>
+        <v>32</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>205</v>
+      </c>
       <c r="F39" s="7"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
-    </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="O39" t="s">
+        <v>22</v>
+      </c>
+      <c r="P39" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>192</v>
+      </c>
+      <c r="R39" t="s">
+        <v>22</v>
+      </c>
+      <c r="S39" t="s">
+        <v>192</v>
+      </c>
+      <c r="T39" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
-        <v>38</v>
-      </c>
-      <c r="D40" s="1"/>
-      <c r="F40" s="7"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
-    </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J40">
+        <f>COUNTIF(E40:I40,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K40">
+        <f>ROUND(J40*10/4,0)</f>
+        <v>10</v>
+      </c>
+      <c r="L40" t="s">
+        <v>22</v>
+      </c>
+      <c r="M40" t="s">
+        <v>22</v>
+      </c>
+      <c r="N40" t="s">
+        <v>22</v>
+      </c>
+      <c r="O40" t="s">
+        <v>22</v>
+      </c>
+      <c r="P40" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>22</v>
+      </c>
+      <c r="R40" t="s">
+        <v>22</v>
+      </c>
+      <c r="S40" t="s">
+        <v>22</v>
+      </c>
+      <c r="T40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
+        <v>28</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>188</v>
+      </c>
       <c r="D41" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="E41" s="1">
+        <v>198</v>
+      </c>
+      <c r="F41" s="7"/>
+      <c r="H41" s="7"/>
+      <c r="I41" s="7"/>
+      <c r="L41" t="s">
+        <v>22</v>
+      </c>
+      <c r="M41" t="s">
+        <v>22</v>
+      </c>
+      <c r="N41" t="s">
+        <v>22</v>
+      </c>
+      <c r="O41" t="s">
+        <v>22</v>
+      </c>
+      <c r="P41" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>22</v>
+      </c>
+      <c r="R41" t="s">
+        <v>22</v>
+      </c>
+      <c r="S41" t="s">
+        <v>192</v>
+      </c>
+      <c r="T41" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
+        <v>40</v>
+      </c>
+      <c r="D42" s="1"/>
+      <c r="F42" s="7"/>
+      <c r="H42" s="7"/>
+      <c r="I42" s="7"/>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
+        <v>41</v>
+      </c>
+      <c r="D43" s="1"/>
+      <c r="F43" s="7"/>
+      <c r="H43" s="7"/>
+      <c r="I43" s="7"/>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="D44" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E44" s="1">
         <f>COUNTIF(E2:E28,"P")</f>
         <v>9</v>
       </c>
-      <c r="F41" s="1">
+      <c r="F44" s="1">
         <f>COUNTIF(F2:F28,"P")</f>
-        <v>6</v>
-      </c>
-      <c r="H41" s="1">
+        <v>7</v>
+      </c>
+      <c r="H44" s="1">
         <f>COUNTIF(H2:H28,"P")</f>
-        <v>7</v>
-      </c>
-      <c r="I41" s="57">
+        <v>5</v>
+      </c>
+      <c r="I44" s="57">
         <f>COUNTIF(I2:I28,"P")</f>
-        <v>3</v>
-      </c>
-      <c r="L41" s="1">
+        <v>4</v>
+      </c>
+      <c r="L44" s="1">
         <f>COUNTIF(L2:L31,"P")</f>
         <v>4</v>
       </c>
-      <c r="M41" s="1">
+      <c r="M44" s="1">
         <f>COUNTIF(M2:M31,"P")</f>
-        <v>3</v>
-      </c>
-      <c r="N41" s="1">
+        <v>4</v>
+      </c>
+      <c r="N44" s="1">
         <f>COUNTIF(N2:N32,"P")</f>
         <v>4</v>
       </c>
-      <c r="O41" s="1">
+      <c r="O44" s="1">
         <f>COUNTIF(O2:O33,"P")</f>
-        <v>5</v>
-      </c>
-      <c r="P41" s="1">
+        <v>4</v>
+      </c>
+      <c r="P44" s="1">
         <f>COUNTIF(P2:P38,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="Q44" s="1">
+        <f>COUNTIF(Q2:Q38,"P")</f>
+        <v>7</v>
+      </c>
+      <c r="R44" s="1">
+        <f>COUNTIF(R2:R38,"P")</f>
         <v>6</v>
       </c>
-      <c r="Q41" s="1">
-        <f>COUNTIF(Q2:Q38,"P")</f>
-        <v>9</v>
-      </c>
-      <c r="R41" s="1">
-        <f>COUNTIF(R2:R38,"P")</f>
-        <v>9</v>
+      <c r="S44" s="1">
+        <f>COUNTIF(S2:S41,"P")</f>
+        <v>8</v>
+      </c>
+      <c r="T44" s="1">
+        <f>COUNTIF(T2:T41,"P")</f>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:R38">
-    <sortCondition ref="R2:R38"/>
-    <sortCondition ref="B2:B38"/>
+  <sortState ref="A2:T41">
+    <sortCondition ref="T2:T41"/>
+    <sortCondition ref="B2:B41"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
agregado de minuta de reunion del 8-10 y modificacion de la list de asistencia
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="222">
   <si>
     <t>Alumnos</t>
   </si>
@@ -4595,7 +4595,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T44"/>
+  <dimension ref="A1:V44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
@@ -4605,10 +4605,10 @@
     <col min="6" max="6" width="11.5703125" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="15.42578125" hidden="1" customWidth="1"/>
     <col min="8" max="10" width="11.5703125" hidden="1" customWidth="1"/>
-    <col min="11" max="12" width="0" hidden="1" customWidth="1"/>
+    <col min="11" max="19" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4669,8 +4669,14 @@
       <c r="T1" s="52">
         <v>46289</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U1" s="52">
+        <v>46296</v>
+      </c>
+      <c r="V1" s="52">
+        <v>46303</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>33</v>
       </c>
@@ -4701,48 +4707,95 @@
       <c r="T2" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U2" t="s">
+        <v>192</v>
+      </c>
+      <c r="V2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>208</v>
+        <v>71</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>217</v>
+        <v>72</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
+        <v>38</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>192</v>
+      </c>
+      <c r="I3" t="s">
+        <v>192</v>
+      </c>
+      <c r="J3">
+        <f>COUNTIF(E3:I3,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K3">
+        <f>ROUND(J3*10/4,0)</f>
+        <v>5</v>
+      </c>
+      <c r="L3" t="s">
+        <v>192</v>
+      </c>
+      <c r="M3" t="s">
+        <v>192</v>
+      </c>
+      <c r="N3" t="s">
+        <v>192</v>
+      </c>
+      <c r="O3" t="s">
+        <v>192</v>
+      </c>
+      <c r="P3" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>192</v>
+      </c>
+      <c r="R3" t="s">
+        <v>192</v>
+      </c>
       <c r="S3" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T3" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U3" t="s">
+        <v>192</v>
+      </c>
+      <c r="V3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>22</v>
+        <v>78</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>192</v>
       </c>
       <c r="H4" t="s">
         <v>192</v>
@@ -4752,11 +4805,11 @@
       </c>
       <c r="J4">
         <f>COUNTIF(E4:I4,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4">
         <f>ROUND(J4*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L4" t="s">
         <v>192</v>
@@ -4785,80 +4838,94 @@
       <c r="T4" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U4" t="s">
+        <v>192</v>
+      </c>
+      <c r="V4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>78</v>
+        <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="H5" t="s">
         <v>192</v>
       </c>
       <c r="I5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="J5">
         <f>COUNTIF(E5:I5,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K5">
         <f>ROUND(J5*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="N5" t="s">
         <v>192</v>
       </c>
       <c r="O5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="P5" t="s">
         <v>192</v>
       </c>
       <c r="Q5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S5" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T5" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="6" spans="1:20" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="U5" t="s">
+        <v>192</v>
+      </c>
+      <c r="V5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>79</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="7" t="s">
         <v>22</v>
       </c>
       <c r="G6"/>
@@ -4866,7 +4933,7 @@
         <v>192</v>
       </c>
       <c r="I6" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="J6">
         <f>COUNTIF(E6:I6,"P")</f>
@@ -4877,65 +4944,68 @@
         <v>5</v>
       </c>
       <c r="L6" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="M6" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="N6" t="s">
         <v>192</v>
       </c>
       <c r="O6" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="P6" t="s">
         <v>192</v>
       </c>
       <c r="Q6" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R6" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="S6" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T6" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I7" t="s">
-        <v>192</v>
-      </c>
+      <c r="U6" t="s">
+        <v>192</v>
+      </c>
+      <c r="V6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A7" s="53">
+        <v>5</v>
+      </c>
+      <c r="B7" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="C7" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D7" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="53"/>
+      <c r="F7" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="G7" s="54" t="s">
+        <v>193</v>
+      </c>
+      <c r="H7" s="54"/>
+      <c r="I7" s="54"/>
       <c r="J7">
         <f>COUNTIF(E7:I7,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7">
         <f>ROUND(J7*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L7" t="s">
         <v>192</v>
@@ -4964,43 +5034,63 @@
       <c r="T7" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U7" t="s">
+        <v>192</v>
+      </c>
+      <c r="V7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>200</v>
+        <v>84</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>201</v>
+        <v>85</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="F8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+        <v>78</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H8" t="s">
+        <v>192</v>
+      </c>
+      <c r="I8" t="s">
+        <v>192</v>
+      </c>
+      <c r="J8">
+        <f>COUNTIF(E8:I8,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <f>ROUND(J8*10/4,0)</f>
+        <v>0</v>
+      </c>
       <c r="L8" t="s">
-        <v>22</v>
-      </c>
-      <c r="M8" t="s">
-        <v>22</v>
+        <v>192</v>
+      </c>
+      <c r="M8" s="54" t="s">
+        <v>192</v>
       </c>
       <c r="N8" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="O8" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="P8" t="s">
         <v>192</v>
       </c>
       <c r="Q8" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R8" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="S8" t="s">
         <v>192</v>
@@ -5008,36 +5098,45 @@
       <c r="T8" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A9" s="53">
-        <v>5</v>
-      </c>
-      <c r="B9" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="C9" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="D9" s="53" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="53"/>
-      <c r="F9" s="53" t="s">
-        <v>192</v>
-      </c>
-      <c r="G9" s="54" t="s">
-        <v>193</v>
-      </c>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="U8" t="s">
+        <v>192</v>
+      </c>
+      <c r="V8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" t="s">
+        <v>192</v>
+      </c>
       <c r="J9">
         <f>COUNTIF(E9:I9,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K9">
         <f>ROUND(J9*10/4,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L9" t="s">
         <v>192</v>
@@ -5066,19 +5165,25 @@
       <c r="T9" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U9" t="s">
+        <v>192</v>
+      </c>
+      <c r="V9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>192</v>
@@ -5100,7 +5205,7 @@
       <c r="L10" t="s">
         <v>192</v>
       </c>
-      <c r="M10" s="54" t="s">
+      <c r="M10" t="s">
         <v>192</v>
       </c>
       <c r="N10" t="s">
@@ -5124,19 +5229,25 @@
       <c r="T10" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U10" t="s">
+        <v>192</v>
+      </c>
+      <c r="V10" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>87</v>
+        <v>186</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>88</v>
+        <v>24</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>22</v>
@@ -5148,73 +5259,82 @@
         <v>22</v>
       </c>
       <c r="I11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="J11">
         <f>COUNTIF(E11:I11,"P")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K11">
         <f>ROUND(J11*10/4,0)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="N11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="O11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="P11" t="s">
         <v>192</v>
       </c>
       <c r="Q11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S11" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T11" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U11" t="s">
+        <v>192</v>
+      </c>
+      <c r="V11" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>90</v>
+        <v>187</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>91</v>
+        <v>188</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H12" t="s">
-        <v>192</v>
-      </c>
-      <c r="I12" t="s">
-        <v>192</v>
+        <v>22</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="J12">
         <f>COUNTIF(E12:I12,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K12">
         <f>ROUND(J12*10/4,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L12" t="s">
         <v>192</v>
@@ -5223,7 +5343,7 @@
         <v>192</v>
       </c>
       <c r="N12" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="O12" t="s">
         <v>192</v>
@@ -5243,120 +5363,133 @@
       <c r="T12" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U12" t="s">
+        <v>192</v>
+      </c>
+      <c r="V12" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>186</v>
+        <v>98</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>24</v>
+        <v>99</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H13" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" t="s">
-        <v>22</v>
+        <v>192</v>
+      </c>
+      <c r="G13" s="56"/>
+      <c r="H13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>192</v>
       </c>
       <c r="J13">
         <f>COUNTIF(E13:I13,"P")</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K13">
         <f>ROUND(J13*10/4,0)</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L13" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="M13" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="N13" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="O13" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="P13" t="s">
         <v>192</v>
       </c>
       <c r="Q13" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R13" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="S13" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T13" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U13" t="s">
+        <v>192</v>
+      </c>
+      <c r="V13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="F14" s="7"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
-      <c r="P14" t="s">
-        <v>22</v>
-      </c>
       <c r="Q14" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R14" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="S14" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T14" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="U14" t="s">
+        <v>22</v>
+      </c>
+      <c r="V14" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>187</v>
+        <v>104</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>188</v>
+        <v>105</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="E15" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F15" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="H15" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H15" s="57" t="s">
         <v>22</v>
       </c>
       <c r="I15" s="7" t="s">
@@ -5371,13 +5504,13 @@
         <v>8</v>
       </c>
       <c r="L15" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M15" t="s">
         <v>192</v>
       </c>
       <c r="N15" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="O15" t="s">
         <v>192</v>
@@ -5392,21 +5525,27 @@
         <v>192</v>
       </c>
       <c r="S15" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T15" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="U15" t="s">
+        <v>192</v>
+      </c>
+      <c r="V15" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>98</v>
+        <v>34</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>99</v>
+        <v>35</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>38</v>
@@ -5414,20 +5553,19 @@
       <c r="F16" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="G16" s="56"/>
       <c r="H16" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>192</v>
       </c>
       <c r="J16">
         <f>COUNTIF(E16:I16,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K16">
         <f>ROUND(J16*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L16" t="s">
         <v>192</v>
@@ -5456,65 +5594,118 @@
       <c r="T16" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U16" t="s">
+        <v>192</v>
+      </c>
+      <c r="V16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>218</v>
+        <v>107</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>219</v>
+        <v>108</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J17">
+        <f>COUNTIF(E17:I17,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <f>ROUND(J17*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L17" t="s">
+        <v>192</v>
+      </c>
+      <c r="M17" t="s">
+        <v>192</v>
+      </c>
+      <c r="N17" t="s">
+        <v>192</v>
+      </c>
+      <c r="O17" t="s">
+        <v>192</v>
+      </c>
+      <c r="P17" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>192</v>
+      </c>
+      <c r="R17" t="s">
+        <v>192</v>
+      </c>
       <c r="S17" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T17" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U17" t="s">
+        <v>192</v>
+      </c>
+      <c r="V17" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>34</v>
+        <v>111</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>194</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="J18">
         <f>COUNTIF(E18:I18,"P")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K18">
         <f>ROUND(J18*10/4,0)</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L18" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M18" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="N18" t="s">
         <v>192</v>
@@ -5537,19 +5728,28 @@
       <c r="T18" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U18" t="s">
+        <v>192</v>
+      </c>
+      <c r="V18" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>17</v>
+        <v>114</v>
+      </c>
+      <c r="D19" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>192</v>
@@ -5562,11 +5762,11 @@
       </c>
       <c r="J19">
         <f>COUNTIF(E19:I19,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19">
         <f>ROUND(J19*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L19" t="s">
         <v>192</v>
@@ -5595,48 +5795,51 @@
       <c r="T19" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U19" t="s">
+        <v>192</v>
+      </c>
+      <c r="V19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>111</v>
+        <v>40</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E20" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="57" t="s">
         <v>22</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="J20">
         <f>COUNTIF(E20:I20,"P")</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K20">
         <f>ROUND(J20*10/4,0)</f>
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L20" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="M20" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="N20" t="s">
         <v>192</v>
@@ -5659,22 +5862,25 @@
       <c r="T20" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U20" t="s">
+        <v>192</v>
+      </c>
+      <c r="V20" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>113</v>
+        <v>49</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D21" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" s="57" t="s">
-        <v>22</v>
+        <v>50</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>192</v>
@@ -5687,11 +5893,11 @@
       </c>
       <c r="J21">
         <f>COUNTIF(E21:I21,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21">
         <f>ROUND(J21*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L21" t="s">
         <v>192</v>
@@ -5720,21 +5926,27 @@
       <c r="T21" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U21" t="s">
+        <v>192</v>
+      </c>
+      <c r="V21" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>117</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D22" s="57" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E22" s="57" t="s">
+      <c r="E22" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F22" s="7" t="s">
@@ -5781,19 +5993,25 @@
       <c r="T22" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U22" t="s">
+        <v>192</v>
+      </c>
+      <c r="V22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>49</v>
+        <v>189</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>50</v>
+        <v>221</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>192</v>
@@ -5839,219 +6057,246 @@
       <c r="T23" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U23" t="s">
+        <v>192</v>
+      </c>
+      <c r="V23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>117</v>
+        <v>202</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>118</v>
+        <v>80</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="N24" t="s">
+        <v>22</v>
+      </c>
+      <c r="O24" t="s">
+        <v>22</v>
+      </c>
+      <c r="P24" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>192</v>
+      </c>
+      <c r="R24" t="s">
+        <v>192</v>
+      </c>
+      <c r="S24" t="s">
+        <v>192</v>
+      </c>
+      <c r="T24" t="s">
+        <v>192</v>
+      </c>
+      <c r="U24" t="s">
+        <v>192</v>
+      </c>
+      <c r="V24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
+        <v>39</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="S25" t="s">
+        <v>22</v>
+      </c>
+      <c r="T25" t="s">
+        <v>192</v>
+      </c>
+      <c r="U25" t="s">
+        <v>192</v>
+      </c>
+      <c r="V25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>22</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H24" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J24">
-        <f>COUNTIF(E24:I24,"P")</f>
+      <c r="E26" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H26" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J26">
+        <f>COUNTIF(E26:I26,"P")</f>
         <v>1</v>
       </c>
-      <c r="K24">
-        <f>ROUND(J24*10/4,0)</f>
+      <c r="K26">
+        <f>ROUND(J26*10/4,0)</f>
         <v>3</v>
       </c>
-      <c r="L24" t="s">
-        <v>192</v>
-      </c>
-      <c r="M24" t="s">
-        <v>192</v>
-      </c>
-      <c r="N24" t="s">
-        <v>192</v>
-      </c>
-      <c r="O24" t="s">
-        <v>192</v>
-      </c>
-      <c r="P24" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>192</v>
-      </c>
-      <c r="R24" t="s">
-        <v>192</v>
-      </c>
-      <c r="S24" t="s">
-        <v>192</v>
-      </c>
-      <c r="T24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>21</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J25">
-        <f>COUNTIF(E25:I25,"P")</f>
+      <c r="L26" t="s">
+        <v>192</v>
+      </c>
+      <c r="M26" t="s">
+        <v>192</v>
+      </c>
+      <c r="N26" t="s">
+        <v>192</v>
+      </c>
+      <c r="O26" t="s">
+        <v>192</v>
+      </c>
+      <c r="P26" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>192</v>
+      </c>
+      <c r="R26" t="s">
+        <v>192</v>
+      </c>
+      <c r="S26" t="s">
+        <v>192</v>
+      </c>
+      <c r="T26" t="s">
+        <v>192</v>
+      </c>
+      <c r="U26" t="s">
+        <v>192</v>
+      </c>
+      <c r="V26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>23</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H27" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J27">
+        <f>COUNTIF(E27:I27,"P")</f>
         <v>0</v>
       </c>
-      <c r="K25">
-        <f>ROUND(J25*10/4,0)</f>
+      <c r="K27">
+        <f>ROUND(J27*10/4,0)</f>
         <v>0</v>
       </c>
-      <c r="L25" t="s">
-        <v>192</v>
-      </c>
-      <c r="M25" t="s">
-        <v>192</v>
-      </c>
-      <c r="N25" t="s">
-        <v>192</v>
-      </c>
-      <c r="O25" t="s">
-        <v>192</v>
-      </c>
-      <c r="P25" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>192</v>
-      </c>
-      <c r="R25" t="s">
-        <v>192</v>
-      </c>
-      <c r="S25" t="s">
-        <v>192</v>
-      </c>
-      <c r="T25" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
-        <v>31</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="N26" t="s">
-        <v>22</v>
-      </c>
-      <c r="O26" t="s">
-        <v>22</v>
-      </c>
-      <c r="P26" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>192</v>
-      </c>
-      <c r="R26" t="s">
-        <v>192</v>
-      </c>
-      <c r="S26" t="s">
-        <v>192</v>
-      </c>
-      <c r="T26" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>39</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
+      <c r="L27" t="s">
+        <v>192</v>
+      </c>
+      <c r="M27" t="s">
+        <v>192</v>
+      </c>
+      <c r="N27" t="s">
+        <v>192</v>
+      </c>
+      <c r="O27" t="s">
+        <v>192</v>
+      </c>
+      <c r="P27" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>192</v>
+      </c>
+      <c r="R27" t="s">
+        <v>192</v>
+      </c>
       <c r="S27" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T27" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U27" t="s">
+        <v>192</v>
+      </c>
+      <c r="V27" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>56</v>
+        <v>132</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>57</v>
+        <v>190</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>192</v>
       </c>
       <c r="J28">
         <f>COUNTIF(E28:I28,"P")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28">
         <f>ROUND(J28*10/4,0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L28" t="s">
         <v>192</v>
@@ -6080,16 +6325,22 @@
       <c r="T28" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U28" t="s">
+        <v>192</v>
+      </c>
+      <c r="V28" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>129</v>
+        <v>64</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>130</v>
+        <v>69</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>53</v>
@@ -6098,18 +6349,18 @@
         <v>192</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>192</v>
       </c>
       <c r="J29">
         <f>COUNTIF(E29:I29,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29">
         <f>ROUND(J29*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L29" t="s">
         <v>192</v>
@@ -6138,16 +6389,22 @@
       <c r="T29" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U29" t="s">
+        <v>192</v>
+      </c>
+      <c r="V29" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>211</v>
@@ -6159,7 +6416,7 @@
         <v>22</v>
       </c>
       <c r="R30" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S30" t="s">
         <v>192</v>
@@ -6167,36 +6424,42 @@
       <c r="T30" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U30" t="s">
+        <v>22</v>
+      </c>
+      <c r="V30" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>190</v>
+        <v>137</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I31" s="7" t="s">
         <v>192</v>
       </c>
       <c r="J31">
         <f>COUNTIF(E31:I31,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K31">
         <f>ROUND(J31*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L31" t="s">
         <v>192</v>
@@ -6225,36 +6488,48 @@
       <c r="T31" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U31" t="s">
+        <v>192</v>
+      </c>
+      <c r="V31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>64</v>
+        <v>139</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>69</v>
+        <v>140</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>53</v>
+        <v>17</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>194</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I32" s="7" t="s">
         <v>192</v>
       </c>
       <c r="J32">
         <f>COUNTIF(E32:I32,"P")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K32">
         <f>ROUND(J32*10/4,0)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L32" t="s">
         <v>192</v>
@@ -6283,16 +6558,22 @@
       <c r="T32" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U32" t="s">
+        <v>192</v>
+      </c>
+      <c r="V32" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>211</v>
@@ -6300,69 +6581,55 @@
       <c r="F33" s="7"/>
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
-      <c r="Q33" t="s">
-        <v>22</v>
-      </c>
-      <c r="R33" t="s">
-        <v>22</v>
-      </c>
       <c r="S33" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T33" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U33" t="s">
+        <v>22</v>
+      </c>
+      <c r="V33" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>136</v>
+        <v>200</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>137</v>
+        <v>201</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J34">
-        <f>COUNTIF(E34:I34,"P")</f>
-        <v>0</v>
-      </c>
-      <c r="K34">
-        <f>ROUND(J34*10/4,0)</f>
-        <v>0</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="F34" s="7"/>
+      <c r="H34" s="7"/>
+      <c r="I34" s="7"/>
       <c r="L34" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M34" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="N34" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="O34" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="P34" t="s">
         <v>192</v>
       </c>
       <c r="Q34" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R34" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S34" t="s">
         <v>192</v>
@@ -6370,104 +6637,84 @@
       <c r="T34" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U34" t="s">
+        <v>22</v>
+      </c>
+      <c r="V34" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>139</v>
+        <v>197</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>140</v>
+        <v>199</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E35" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>194</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J35">
-        <f>COUNTIF(E35:I35,"P")</f>
-        <v>2</v>
-      </c>
-      <c r="K35">
-        <f>ROUND(J35*10/4,0)</f>
-        <v>5</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="F35" s="7"/>
+      <c r="H35" s="7"/>
+      <c r="I35" s="7"/>
       <c r="L35" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M35" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="N35" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="O35" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="P35" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="Q35" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R35" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S35" t="s">
         <v>192</v>
       </c>
       <c r="T35" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="U35" t="s">
+        <v>22</v>
+      </c>
+      <c r="V35" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="F36" s="7"/>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
-      <c r="L36" t="s">
-        <v>22</v>
-      </c>
-      <c r="M36" t="s">
-        <v>22</v>
-      </c>
-      <c r="N36" t="s">
-        <v>22</v>
-      </c>
-      <c r="O36" t="s">
-        <v>22</v>
-      </c>
       <c r="P36" t="s">
         <v>22</v>
       </c>
       <c r="Q36" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R36" t="s">
         <v>22</v>
@@ -6476,18 +6723,24 @@
         <v>192</v>
       </c>
       <c r="T36" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="U36" t="s">
+        <v>192</v>
+      </c>
+      <c r="V36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>211</v>
@@ -6495,96 +6748,102 @@
       <c r="F37" s="7"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
-      <c r="Q37" t="s">
-        <v>22</v>
-      </c>
-      <c r="R37" t="s">
-        <v>192</v>
-      </c>
       <c r="S37" t="s">
         <v>22</v>
       </c>
       <c r="T37" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="U37" t="s">
+        <v>192</v>
+      </c>
+      <c r="V37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>104</v>
+        <v>203</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>105</v>
+        <v>204</v>
       </c>
       <c r="D38" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F38" s="7"/>
+      <c r="H38" s="7"/>
+      <c r="I38" s="7"/>
+      <c r="O38" t="s">
+        <v>22</v>
+      </c>
+      <c r="P38" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>192</v>
+      </c>
+      <c r="R38" t="s">
+        <v>22</v>
+      </c>
+      <c r="S38" t="s">
+        <v>192</v>
+      </c>
+      <c r="T38" t="s">
+        <v>22</v>
+      </c>
+      <c r="U38" t="s">
+        <v>22</v>
+      </c>
+      <c r="V38" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
+        <v>18</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E38" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H38" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J38">
-        <f>COUNTIF(E38:I38,"P")</f>
-        <v>3</v>
-      </c>
-      <c r="K38">
-        <f>ROUND(J38*10/4,0)</f>
-        <v>8</v>
-      </c>
-      <c r="L38" t="s">
-        <v>22</v>
-      </c>
-      <c r="M38" t="s">
-        <v>192</v>
-      </c>
-      <c r="N38" t="s">
-        <v>192</v>
-      </c>
-      <c r="O38" t="s">
-        <v>192</v>
-      </c>
-      <c r="P38" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>192</v>
-      </c>
-      <c r="R38" t="s">
-        <v>192</v>
-      </c>
-      <c r="S38" t="s">
-        <v>22</v>
-      </c>
-      <c r="T38" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A39" s="1">
-        <v>32</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="F39" s="7"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="7"/>
+      <c r="E39" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H39" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J39">
+        <f>COUNTIF(E39:I39,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K39">
+        <f>ROUND(J39*10/4,0)</f>
+        <v>10</v>
+      </c>
+      <c r="L39" t="s">
+        <v>22</v>
+      </c>
+      <c r="M39" t="s">
+        <v>22</v>
+      </c>
+      <c r="N39" t="s">
+        <v>22</v>
+      </c>
       <c r="O39" t="s">
         <v>22</v>
       </c>
@@ -6592,51 +6851,40 @@
         <v>22</v>
       </c>
       <c r="Q39" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R39" t="s">
         <v>22</v>
       </c>
       <c r="S39" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T39" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U39" t="s">
+        <v>22</v>
+      </c>
+      <c r="V39" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>189</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>47</v>
+        <v>188</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J40">
-        <f>COUNTIF(E40:I40,"P")</f>
-        <v>4</v>
-      </c>
-      <c r="K40">
-        <f>ROUND(J40*10/4,0)</f>
-        <v>10</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="F40" s="7"/>
+      <c r="H40" s="7"/>
+      <c r="I40" s="7"/>
       <c r="L40" t="s">
         <v>22</v>
       </c>
@@ -6659,57 +6907,54 @@
         <v>22</v>
       </c>
       <c r="S40" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T40" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U40" t="s">
+        <v>22</v>
+      </c>
+      <c r="V40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>189</v>
+        <v>213</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>188</v>
+        <v>214</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="F41" s="7"/>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
-      <c r="L41" t="s">
-        <v>22</v>
-      </c>
-      <c r="M41" t="s">
-        <v>22</v>
-      </c>
-      <c r="N41" t="s">
-        <v>22</v>
-      </c>
-      <c r="O41" t="s">
-        <v>22</v>
-      </c>
-      <c r="P41" t="s">
-        <v>22</v>
-      </c>
       <c r="Q41" t="s">
         <v>22</v>
       </c>
       <c r="R41" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="S41" t="s">
         <v>192</v>
       </c>
       <c r="T41" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="U41" t="s">
+        <v>192</v>
+      </c>
+      <c r="V41" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -6718,7 +6963,7 @@
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -6726,26 +6971,27 @@
       <c r="F43" s="7"/>
       <c r="H43" s="7"/>
       <c r="I43" s="7"/>
-    </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="V43" s="56"/>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
       <c r="D44" s="1" t="s">
         <v>191</v>
       </c>
       <c r="E44" s="1">
         <f>COUNTIF(E2:E28,"P")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F44" s="1">
         <f>COUNTIF(F2:F28,"P")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H44" s="1">
         <f>COUNTIF(H2:H28,"P")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I44" s="57">
         <f>COUNTIF(I2:I28,"P")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L44" s="1">
         <f>COUNTIF(L2:L31,"P")</f>
@@ -6753,27 +6999,27 @@
       </c>
       <c r="M44" s="1">
         <f>COUNTIF(M2:M31,"P")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N44" s="1">
         <f>COUNTIF(N2:N32,"P")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O44" s="1">
         <f>COUNTIF(O2:O33,"P")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P44" s="1">
         <f>COUNTIF(P2:P38,"P")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q44" s="1">
         <f>COUNTIF(Q2:Q38,"P")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="R44" s="1">
         <f>COUNTIF(R2:R38,"P")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S44" s="1">
         <f>COUNTIF(S2:S41,"P")</f>
@@ -6783,10 +7029,18 @@
         <f>COUNTIF(T2:T41,"P")</f>
         <v>6</v>
       </c>
+      <c r="U44" s="1">
+        <f>COUNTIF(U2:U41,"P")</f>
+        <v>8</v>
+      </c>
+      <c r="V44" s="1">
+        <f>COUNTIF(V2:V41,"P")</f>
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:T41">
-    <sortCondition ref="T2:T41"/>
+  <sortState ref="A2:V41">
+    <sortCondition ref="V2:V41"/>
     <sortCondition ref="B2:B41"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>

<commit_message>
agregado de minuta del 15-10
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="alumnos" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="222">
   <si>
     <t>Alumnos</t>
   </si>
@@ -627,9 +627,6 @@
     <t>Salvador</t>
   </si>
   <si>
-    <t>Barzo Marchi</t>
-  </si>
-  <si>
     <t>Juan</t>
   </si>
   <si>
@@ -691,6 +688,9 @@
   </si>
   <si>
     <t>Fabrizio</t>
+  </si>
+  <si>
+    <t>Bazo Marchi</t>
   </si>
 </sst>
 </file>
@@ -4595,7 +4595,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:W44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
@@ -4608,7 +4608,7 @@
     <col min="11" max="19" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4675,19 +4675,22 @@
       <c r="V1" s="52">
         <v>46303</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W1" s="52">
+        <v>46310</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>209</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F2" s="7"/>
       <c r="H2" s="7"/>
@@ -4713,8 +4716,11 @@
       <c r="V2" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -4780,8 +4786,11 @@
       <c r="V3" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -4844,8 +4853,11 @@
       <c r="V4" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -4908,8 +4920,11 @@
       <c r="V5" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="W5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -4976,8 +4991,11 @@
       <c r="V6" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" s="53">
         <v>5</v>
       </c>
@@ -5040,8 +5058,11 @@
       <c r="V7" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -5104,8 +5125,11 @@
       <c r="V8" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -5171,8 +5195,11 @@
       <c r="V9" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -5235,8 +5262,11 @@
       <c r="V10" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W10" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -5302,175 +5332,190 @@
       <c r="V11" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W11" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
+        <v>32</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="P12" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>192</v>
+      </c>
+      <c r="R12" t="s">
+        <v>22</v>
+      </c>
+      <c r="S12" t="s">
+        <v>192</v>
+      </c>
+      <c r="T12" t="s">
+        <v>192</v>
+      </c>
+      <c r="U12" t="s">
+        <v>192</v>
+      </c>
+      <c r="V12" t="s">
+        <v>22</v>
+      </c>
+      <c r="W12" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="7" t="s">
+      <c r="F13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="H12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J12">
-        <f>COUNTIF(E12:I12,"P")</f>
-        <v>3</v>
-      </c>
-      <c r="K12">
-        <f>ROUND(J12*10/4,0)</f>
-        <v>8</v>
-      </c>
-      <c r="L12" t="s">
-        <v>192</v>
-      </c>
-      <c r="M12" t="s">
-        <v>192</v>
-      </c>
-      <c r="N12" t="s">
-        <v>22</v>
-      </c>
-      <c r="O12" t="s">
-        <v>192</v>
-      </c>
-      <c r="P12" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>192</v>
-      </c>
-      <c r="R12" t="s">
-        <v>192</v>
-      </c>
-      <c r="S12" t="s">
-        <v>192</v>
-      </c>
-      <c r="T12" t="s">
-        <v>192</v>
-      </c>
-      <c r="U12" t="s">
-        <v>192</v>
-      </c>
-      <c r="V12" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
-        <v>11</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="G13" s="56"/>
       <c r="H13" s="7" t="s">
         <v>22</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="J13">
         <f>COUNTIF(E13:I13,"P")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K13">
         <f>ROUND(J13*10/4,0)</f>
+        <v>8</v>
+      </c>
+      <c r="L13" t="s">
+        <v>192</v>
+      </c>
+      <c r="M13" t="s">
+        <v>192</v>
+      </c>
+      <c r="N13" t="s">
+        <v>22</v>
+      </c>
+      <c r="O13" t="s">
+        <v>192</v>
+      </c>
+      <c r="P13" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>192</v>
+      </c>
+      <c r="R13" t="s">
+        <v>192</v>
+      </c>
+      <c r="S13" t="s">
+        <v>192</v>
+      </c>
+      <c r="T13" t="s">
+        <v>192</v>
+      </c>
+      <c r="U13" t="s">
+        <v>192</v>
+      </c>
+      <c r="V13" t="s">
+        <v>192</v>
+      </c>
+      <c r="W13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>11</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="G14" s="56"/>
+      <c r="H14" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J14">
+        <f>COUNTIF(E14:I14,"P")</f>
+        <v>1</v>
+      </c>
+      <c r="K14">
+        <f>ROUND(J14*10/4,0)</f>
         <v>3</v>
       </c>
-      <c r="L13" t="s">
-        <v>192</v>
-      </c>
-      <c r="M13" t="s">
-        <v>192</v>
-      </c>
-      <c r="N13" t="s">
-        <v>192</v>
-      </c>
-      <c r="O13" t="s">
-        <v>192</v>
-      </c>
-      <c r="P13" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>192</v>
-      </c>
-      <c r="R13" t="s">
-        <v>192</v>
-      </c>
-      <c r="S13" t="s">
-        <v>192</v>
-      </c>
-      <c r="T13" t="s">
-        <v>192</v>
-      </c>
-      <c r="U13" t="s">
-        <v>192</v>
-      </c>
-      <c r="V13" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A14" s="1">
-        <v>34</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
+      <c r="L14" t="s">
+        <v>192</v>
+      </c>
+      <c r="M14" t="s">
+        <v>192</v>
+      </c>
+      <c r="N14" t="s">
+        <v>192</v>
+      </c>
+      <c r="O14" t="s">
+        <v>192</v>
+      </c>
+      <c r="P14" t="s">
+        <v>192</v>
+      </c>
       <c r="Q14" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R14" t="s">
         <v>192</v>
       </c>
       <c r="S14" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T14" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="U14" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="V14" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W14" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>12</v>
       </c>
@@ -5536,83 +5581,54 @@
       <c r="V15" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W15" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
+        <v>38</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="S16" t="s">
+        <v>22</v>
+      </c>
+      <c r="T16" t="s">
+        <v>192</v>
+      </c>
+      <c r="U16" t="s">
+        <v>192</v>
+      </c>
+      <c r="V16" t="s">
+        <v>22</v>
+      </c>
+      <c r="W16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>13</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D17" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J16">
-        <f>COUNTIF(E16:I16,"P")</f>
-        <v>0</v>
-      </c>
-      <c r="K16">
-        <f>ROUND(J16*10/4,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L16" t="s">
-        <v>192</v>
-      </c>
-      <c r="M16" t="s">
-        <v>192</v>
-      </c>
-      <c r="N16" t="s">
-        <v>192</v>
-      </c>
-      <c r="O16" t="s">
-        <v>192</v>
-      </c>
-      <c r="P16" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>192</v>
-      </c>
-      <c r="R16" t="s">
-        <v>192</v>
-      </c>
-      <c r="S16" t="s">
-        <v>192</v>
-      </c>
-      <c r="T16" t="s">
-        <v>192</v>
-      </c>
-      <c r="U16" t="s">
-        <v>192</v>
-      </c>
-      <c r="V16" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A17" s="1">
-        <v>14</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>192</v>
@@ -5664,48 +5680,45 @@
       <c r="V17" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W17" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>57</v>
+        <v>108</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F18" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="J18">
         <f>COUNTIF(E18:I18,"P")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K18">
         <f>ROUND(J18*10/4,0)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="M18" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="N18" t="s">
         <v>192</v>
@@ -5734,45 +5747,51 @@
       <c r="V18" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W18" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D19" s="57" t="s">
-        <v>38</v>
-      </c>
-      <c r="E19" s="57" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E19" s="7" t="s">
         <v>22</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>194</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="J19">
         <f>COUNTIF(E19:I19,"P")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K19">
         <f>ROUND(J19*10/4,0)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L19" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M19" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="N19" t="s">
         <v>192</v>
@@ -5801,16 +5820,19 @@
       <c r="V19" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>40</v>
+        <v>113</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>41</v>
+        <v>114</v>
       </c>
       <c r="D20" s="57" t="s">
         <v>38</v>
@@ -5868,19 +5890,25 @@
       <c r="V20" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W20" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>53</v>
+        <v>41</v>
+      </c>
+      <c r="D21" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="57" t="s">
+        <v>22</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>192</v>
@@ -5893,11 +5921,11 @@
       </c>
       <c r="J21">
         <f>COUNTIF(E21:I21,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21">
         <f>ROUND(J21*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L21" t="s">
         <v>192</v>
@@ -5932,22 +5960,22 @@
       <c r="V21" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W21" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>117</v>
+        <v>49</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>192</v>
@@ -5960,11 +5988,11 @@
       </c>
       <c r="J22">
         <f>COUNTIF(E22:I22,"P")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22">
         <f>ROUND(J22*10/4,0)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L22" t="s">
         <v>192</v>
@@ -5999,20 +6027,26 @@
       <c r="V22" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>189</v>
+        <v>117</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>221</v>
+        <v>118</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="E23" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F23" s="7" t="s">
         <v>192</v>
       </c>
@@ -6024,108 +6058,149 @@
       </c>
       <c r="J23">
         <f>COUNTIF(E23:I23,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23">
         <f>ROUND(J23*10/4,0)</f>
+        <v>3</v>
+      </c>
+      <c r="L23" t="s">
+        <v>192</v>
+      </c>
+      <c r="M23" t="s">
+        <v>192</v>
+      </c>
+      <c r="N23" t="s">
+        <v>192</v>
+      </c>
+      <c r="O23" t="s">
+        <v>192</v>
+      </c>
+      <c r="P23" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>192</v>
+      </c>
+      <c r="R23" t="s">
+        <v>192</v>
+      </c>
+      <c r="S23" t="s">
+        <v>192</v>
+      </c>
+      <c r="T23" t="s">
+        <v>192</v>
+      </c>
+      <c r="U23" t="s">
+        <v>192</v>
+      </c>
+      <c r="V23" t="s">
+        <v>192</v>
+      </c>
+      <c r="W23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>21</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H24" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J24">
+        <f>COUNTIF(E24:I24,"P")</f>
         <v>0</v>
       </c>
-      <c r="L23" t="s">
-        <v>192</v>
-      </c>
-      <c r="M23" t="s">
-        <v>192</v>
-      </c>
-      <c r="N23" t="s">
-        <v>192</v>
-      </c>
-      <c r="O23" t="s">
-        <v>192</v>
-      </c>
-      <c r="P23" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q23" t="s">
-        <v>192</v>
-      </c>
-      <c r="R23" t="s">
-        <v>192</v>
-      </c>
-      <c r="S23" t="s">
-        <v>192</v>
-      </c>
-      <c r="T23" t="s">
-        <v>192</v>
-      </c>
-      <c r="U23" t="s">
-        <v>192</v>
-      </c>
-      <c r="V23" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
+      <c r="K24">
+        <f>ROUND(J24*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L24" t="s">
+        <v>192</v>
+      </c>
+      <c r="M24" t="s">
+        <v>192</v>
+      </c>
+      <c r="N24" t="s">
+        <v>192</v>
+      </c>
+      <c r="O24" t="s">
+        <v>192</v>
+      </c>
+      <c r="P24" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>192</v>
+      </c>
+      <c r="R24" t="s">
+        <v>192</v>
+      </c>
+      <c r="S24" t="s">
+        <v>192</v>
+      </c>
+      <c r="T24" t="s">
+        <v>192</v>
+      </c>
+      <c r="U24" t="s">
+        <v>192</v>
+      </c>
+      <c r="V24" t="s">
+        <v>192</v>
+      </c>
+      <c r="W24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
         <v>31</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>202</v>
-      </c>
-      <c r="C24" s="1" t="s">
+      <c r="B25" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D25" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="F24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="N24" t="s">
-        <v>22</v>
-      </c>
-      <c r="O24" t="s">
-        <v>22</v>
-      </c>
-      <c r="P24" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>192</v>
-      </c>
-      <c r="R24" t="s">
-        <v>192</v>
-      </c>
-      <c r="S24" t="s">
-        <v>192</v>
-      </c>
-      <c r="T24" t="s">
-        <v>192</v>
-      </c>
-      <c r="U24" t="s">
-        <v>192</v>
-      </c>
-      <c r="V24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
-        <v>39</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>211</v>
       </c>
       <c r="F25" s="7"/>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
+      <c r="N25" t="s">
+        <v>22</v>
+      </c>
+      <c r="O25" t="s">
+        <v>22</v>
+      </c>
+      <c r="P25" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>192</v>
+      </c>
+      <c r="R25" t="s">
+        <v>192</v>
+      </c>
       <c r="S25" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T25" t="s">
         <v>192</v>
@@ -6136,86 +6211,57 @@
       <c r="V25" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B26" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="S26" t="s">
+        <v>22</v>
+      </c>
+      <c r="T26" t="s">
+        <v>192</v>
+      </c>
+      <c r="U26" t="s">
+        <v>192</v>
+      </c>
+      <c r="V26" t="s">
+        <v>192</v>
+      </c>
+      <c r="W26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
+        <v>22</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E26" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H26" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J26">
-        <f>COUNTIF(E26:I26,"P")</f>
-        <v>1</v>
-      </c>
-      <c r="K26">
-        <f>ROUND(J26*10/4,0)</f>
-        <v>3</v>
-      </c>
-      <c r="L26" t="s">
-        <v>192</v>
-      </c>
-      <c r="M26" t="s">
-        <v>192</v>
-      </c>
-      <c r="N26" t="s">
-        <v>192</v>
-      </c>
-      <c r="O26" t="s">
-        <v>192</v>
-      </c>
-      <c r="P26" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>192</v>
-      </c>
-      <c r="R26" t="s">
-        <v>192</v>
-      </c>
-      <c r="S26" t="s">
-        <v>192</v>
-      </c>
-      <c r="T26" t="s">
-        <v>192</v>
-      </c>
-      <c r="U26" t="s">
-        <v>192</v>
-      </c>
-      <c r="V26" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
-        <v>23</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>53</v>
+      <c r="E27" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>192</v>
@@ -6228,11 +6274,11 @@
       </c>
       <c r="J27">
         <f>COUNTIF(E27:I27,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27">
         <f>ROUND(J27*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L27" t="s">
         <v>192</v>
@@ -6267,199 +6313,211 @@
       <c r="V27" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W27" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>192</v>
       </c>
       <c r="J28">
         <f>COUNTIF(E28:I28,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K28">
         <f>ROUND(J28*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L28" t="s">
+        <v>192</v>
+      </c>
+      <c r="M28" t="s">
+        <v>192</v>
+      </c>
+      <c r="N28" t="s">
+        <v>192</v>
+      </c>
+      <c r="O28" t="s">
+        <v>192</v>
+      </c>
+      <c r="P28" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>192</v>
+      </c>
+      <c r="R28" t="s">
+        <v>192</v>
+      </c>
+      <c r="S28" t="s">
+        <v>192</v>
+      </c>
+      <c r="T28" t="s">
+        <v>192</v>
+      </c>
+      <c r="U28" t="s">
+        <v>192</v>
+      </c>
+      <c r="V28" t="s">
+        <v>192</v>
+      </c>
+      <c r="W28" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>35</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F29" s="7"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="Q29" t="s">
+        <v>22</v>
+      </c>
+      <c r="R29" t="s">
+        <v>192</v>
+      </c>
+      <c r="S29" t="s">
+        <v>192</v>
+      </c>
+      <c r="T29" t="s">
+        <v>192</v>
+      </c>
+      <c r="U29" t="s">
+        <v>192</v>
+      </c>
+      <c r="V29" t="s">
+        <v>22</v>
+      </c>
+      <c r="W29" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
+        <v>24</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J30">
+        <f>COUNTIF(E30:I30,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K30">
+        <f>ROUND(J30*10/4,0)</f>
         <v>5</v>
       </c>
-      <c r="L28" t="s">
-        <v>192</v>
-      </c>
-      <c r="M28" t="s">
-        <v>192</v>
-      </c>
-      <c r="N28" t="s">
-        <v>192</v>
-      </c>
-      <c r="O28" t="s">
-        <v>192</v>
-      </c>
-      <c r="P28" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>192</v>
-      </c>
-      <c r="R28" t="s">
-        <v>192</v>
-      </c>
-      <c r="S28" t="s">
-        <v>192</v>
-      </c>
-      <c r="T28" t="s">
-        <v>192</v>
-      </c>
-      <c r="U28" t="s">
-        <v>192</v>
-      </c>
-      <c r="V28" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
+      <c r="L30" t="s">
+        <v>192</v>
+      </c>
+      <c r="M30" t="s">
+        <v>192</v>
+      </c>
+      <c r="N30" t="s">
+        <v>192</v>
+      </c>
+      <c r="O30" t="s">
+        <v>192</v>
+      </c>
+      <c r="P30" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>192</v>
+      </c>
+      <c r="R30" t="s">
+        <v>192</v>
+      </c>
+      <c r="S30" t="s">
+        <v>192</v>
+      </c>
+      <c r="T30" t="s">
+        <v>192</v>
+      </c>
+      <c r="U30" t="s">
+        <v>192</v>
+      </c>
+      <c r="V30" t="s">
+        <v>192</v>
+      </c>
+      <c r="W30" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
         <v>25</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J29">
-        <f>COUNTIF(E29:I29,"P")</f>
-        <v>1</v>
-      </c>
-      <c r="K29">
-        <f>ROUND(J29*10/4,0)</f>
-        <v>3</v>
-      </c>
-      <c r="L29" t="s">
-        <v>192</v>
-      </c>
-      <c r="M29" t="s">
-        <v>192</v>
-      </c>
-      <c r="N29" t="s">
-        <v>192</v>
-      </c>
-      <c r="O29" t="s">
-        <v>192</v>
-      </c>
-      <c r="P29" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>192</v>
-      </c>
-      <c r="R29" t="s">
-        <v>192</v>
-      </c>
-      <c r="S29" t="s">
-        <v>192</v>
-      </c>
-      <c r="T29" t="s">
-        <v>192</v>
-      </c>
-      <c r="U29" t="s">
-        <v>192</v>
-      </c>
-      <c r="V29" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
-        <v>36</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F30" s="7"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
-      <c r="Q30" t="s">
-        <v>22</v>
-      </c>
-      <c r="R30" t="s">
-        <v>22</v>
-      </c>
-      <c r="S30" t="s">
-        <v>192</v>
-      </c>
-      <c r="T30" t="s">
-        <v>192</v>
-      </c>
-      <c r="U30" t="s">
-        <v>22</v>
-      </c>
-      <c r="V30" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A31" s="1">
-        <v>26</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>38</v>
-      </c>
       <c r="F31" s="7" t="s">
         <v>192</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="I31" s="7" t="s">
         <v>192</v>
       </c>
       <c r="J31">
         <f>COUNTIF(E31:I31,"P")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31">
         <f>ROUND(J31*10/4,0)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L31" t="s">
         <v>192</v>
@@ -6494,28 +6552,25 @@
       <c r="V31" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E32" s="7" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>192</v>
@@ -6525,114 +6580,140 @@
       </c>
       <c r="J32">
         <f>COUNTIF(E32:I32,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K32">
         <f>ROUND(J32*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L32" t="s">
+        <v>192</v>
+      </c>
+      <c r="M32" t="s">
+        <v>192</v>
+      </c>
+      <c r="N32" t="s">
+        <v>192</v>
+      </c>
+      <c r="O32" t="s">
+        <v>192</v>
+      </c>
+      <c r="P32" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>192</v>
+      </c>
+      <c r="R32" t="s">
+        <v>192</v>
+      </c>
+      <c r="S32" t="s">
+        <v>192</v>
+      </c>
+      <c r="T32" t="s">
+        <v>192</v>
+      </c>
+      <c r="U32" t="s">
+        <v>192</v>
+      </c>
+      <c r="V32" t="s">
+        <v>192</v>
+      </c>
+      <c r="W32" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
+        <v>27</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J33">
+        <f>COUNTIF(E33:I33,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K33">
+        <f>ROUND(J33*10/4,0)</f>
         <v>5</v>
       </c>
-      <c r="L32" t="s">
-        <v>192</v>
-      </c>
-      <c r="M32" t="s">
-        <v>192</v>
-      </c>
-      <c r="N32" t="s">
-        <v>192</v>
-      </c>
-      <c r="O32" t="s">
-        <v>192</v>
-      </c>
-      <c r="P32" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>192</v>
-      </c>
-      <c r="R32" t="s">
-        <v>192</v>
-      </c>
-      <c r="S32" t="s">
-        <v>192</v>
-      </c>
-      <c r="T32" t="s">
-        <v>192</v>
-      </c>
-      <c r="U32" t="s">
-        <v>192</v>
-      </c>
-      <c r="V32" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A33" s="1">
+      <c r="L33" t="s">
+        <v>192</v>
+      </c>
+      <c r="M33" t="s">
+        <v>192</v>
+      </c>
+      <c r="N33" t="s">
+        <v>192</v>
+      </c>
+      <c r="O33" t="s">
+        <v>192</v>
+      </c>
+      <c r="P33" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>192</v>
+      </c>
+      <c r="R33" t="s">
+        <v>192</v>
+      </c>
+      <c r="S33" t="s">
+        <v>192</v>
+      </c>
+      <c r="T33" t="s">
+        <v>192</v>
+      </c>
+      <c r="U33" t="s">
+        <v>192</v>
+      </c>
+      <c r="V33" t="s">
+        <v>192</v>
+      </c>
+      <c r="W33" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
         <v>37</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="F33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="S33" t="s">
-        <v>22</v>
-      </c>
-      <c r="T33" t="s">
-        <v>192</v>
-      </c>
-      <c r="U33" t="s">
-        <v>22</v>
-      </c>
-      <c r="V33" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A34" s="1">
-        <v>30</v>
-      </c>
       <c r="B34" s="1" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="F34" s="7"/>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
-      <c r="L34" t="s">
-        <v>22</v>
-      </c>
-      <c r="M34" t="s">
-        <v>22</v>
-      </c>
-      <c r="N34" t="s">
-        <v>22</v>
-      </c>
-      <c r="O34" t="s">
-        <v>22</v>
-      </c>
-      <c r="P34" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>22</v>
-      </c>
-      <c r="R34" t="s">
-        <v>22</v>
-      </c>
       <c r="S34" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T34" t="s">
         <v>192</v>
@@ -6643,16 +6724,19 @@
       <c r="V34" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W34" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>197</v>
+        <v>221</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>198</v>
@@ -6673,7 +6757,7 @@
         <v>22</v>
       </c>
       <c r="P35" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="Q35" t="s">
         <v>22</v>
@@ -6685,7 +6769,7 @@
         <v>192</v>
       </c>
       <c r="T35" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="U35" t="s">
         <v>22</v>
@@ -6693,28 +6777,43 @@
       <c r="V35" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W35" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="F36" s="7"/>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
+      <c r="L36" t="s">
+        <v>22</v>
+      </c>
+      <c r="M36" t="s">
+        <v>22</v>
+      </c>
+      <c r="N36" t="s">
+        <v>22</v>
+      </c>
+      <c r="O36" t="s">
+        <v>22</v>
+      </c>
       <c r="P36" t="s">
         <v>22</v>
       </c>
       <c r="Q36" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R36" t="s">
         <v>22</v>
@@ -6723,56 +6822,68 @@
         <v>192</v>
       </c>
       <c r="T36" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="U36" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="V36" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F37" s="7"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
+      <c r="Q37" t="s">
+        <v>22</v>
+      </c>
+      <c r="R37" t="s">
+        <v>192</v>
+      </c>
       <c r="S37" t="s">
         <v>22</v>
       </c>
       <c r="T37" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="U37" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="V37" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="W37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>32</v>
       </c>
       <c r="B38" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="C38" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="F38" s="7"/>
       <c r="H38" s="7"/>
@@ -6801,8 +6912,11 @@
       <c r="V38" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W38" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>18</v>
       </c>
@@ -6868,8 +6982,11 @@
       <c r="V39" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W39" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>28</v>
       </c>
@@ -6918,19 +7035,22 @@
       <c r="V40" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F41" s="7"/>
       <c r="H41" s="7"/>
@@ -6939,7 +7059,7 @@
         <v>22</v>
       </c>
       <c r="R41" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S41" t="s">
         <v>192</v>
@@ -6948,13 +7068,16 @@
         <v>192</v>
       </c>
       <c r="U41" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="V41" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="W41" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -6963,7 +7086,7 @@
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -6973,7 +7096,7 @@
       <c r="I43" s="7"/>
       <c r="V43" s="56"/>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="D44" s="1" t="s">
         <v>191</v>
       </c>
@@ -6983,11 +7106,11 @@
       </c>
       <c r="F44" s="1">
         <f>COUNTIF(F2:F28,"P")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H44" s="1">
         <f>COUNTIF(H2:H28,"P")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I44" s="57">
         <f>COUNTIF(I2:I28,"P")</f>
@@ -7019,7 +7142,7 @@
       </c>
       <c r="R44" s="1">
         <f>COUNTIF(R2:R38,"P")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S44" s="1">
         <f>COUNTIF(S2:S41,"P")</f>
@@ -7037,10 +7160,14 @@
         <f>COUNTIF(V2:V41,"P")</f>
         <v>9</v>
       </c>
+      <c r="W44" s="1">
+        <f>COUNTIF(W2:W41,"P")</f>
+        <v>8</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:V41">
-    <sortCondition ref="V2:V41"/>
+  <sortState ref="A2:W41">
+    <sortCondition ref="W2:W41"/>
     <sortCondition ref="B2:B41"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>

<commit_message>
agregado de minuta de 29-10 -startup
</commit_message>
<xml_diff>
--- a/documentacion/generada/ListaAlumnosYdocentes.xlsx
+++ b/documentacion/generada/ListaAlumnosYdocentes.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="alumnos" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1012" uniqueCount="222">
   <si>
     <t>Alumnos</t>
   </si>
@@ -4595,20 +4595,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W44"/>
+  <dimension ref="A1:X44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="20.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" style="1" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="11.5703125" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="15.42578125" hidden="1" customWidth="1"/>
     <col min="8" max="10" width="11.5703125" hidden="1" customWidth="1"/>
-    <col min="11" max="19" width="0" hidden="1" customWidth="1"/>
+    <col min="11" max="21" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -4678,8 +4678,11 @@
       <c r="W1" s="52">
         <v>46310</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X1" s="52">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>33</v>
       </c>
@@ -4719,92 +4722,63 @@
       <c r="W2" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
+        <v>37</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="S3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" t="s">
+        <v>192</v>
+      </c>
+      <c r="U3" t="s">
+        <v>22</v>
+      </c>
+      <c r="V3" t="s">
+        <v>22</v>
+      </c>
+      <c r="W3" t="s">
+        <v>22</v>
+      </c>
+      <c r="X3" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>192</v>
-      </c>
-      <c r="I3" t="s">
-        <v>192</v>
-      </c>
-      <c r="J3">
-        <f>COUNTIF(E3:I3,"P")</f>
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <f>ROUND(J3*10/4,0)</f>
-        <v>5</v>
-      </c>
-      <c r="L3" t="s">
-        <v>192</v>
-      </c>
-      <c r="M3" t="s">
-        <v>192</v>
-      </c>
-      <c r="N3" t="s">
-        <v>192</v>
-      </c>
-      <c r="O3" t="s">
-        <v>192</v>
-      </c>
-      <c r="P3" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>192</v>
-      </c>
-      <c r="R3" t="s">
-        <v>192</v>
-      </c>
-      <c r="S3" t="s">
-        <v>192</v>
-      </c>
-      <c r="T3" t="s">
-        <v>192</v>
-      </c>
-      <c r="U3" t="s">
-        <v>192</v>
-      </c>
-      <c r="V3" t="s">
-        <v>192</v>
-      </c>
-      <c r="W3" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>192</v>
+      <c r="E4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="H4" t="s">
         <v>192</v>
@@ -4814,11 +4788,11 @@
       </c>
       <c r="J4">
         <f>COUNTIF(E4:I4,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4">
         <f>ROUND(J4*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L4" t="s">
         <v>192</v>
@@ -4856,60 +4830,63 @@
       <c r="W4" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X4" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>75</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>76</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="H5" t="s">
         <v>192</v>
       </c>
       <c r="I5" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="J5">
         <f>COUNTIF(E5:I5,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <f>ROUND(J5*10/4,0)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="M5" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="N5" t="s">
         <v>192</v>
       </c>
       <c r="O5" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="P5" t="s">
         <v>192</v>
       </c>
       <c r="Q5" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R5" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="S5" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T5" t="s">
         <v>192</v>
@@ -4923,24 +4900,25 @@
       <c r="W5" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="6" spans="1:23" s="54" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="X5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" s="54" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1" t="s">
         <v>22</v>
       </c>
       <c r="G6"/>
@@ -4948,7 +4926,7 @@
         <v>192</v>
       </c>
       <c r="I6" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="J6">
         <f>COUNTIF(E6:I6,"P")</f>
@@ -4959,28 +4937,28 @@
         <v>5</v>
       </c>
       <c r="L6" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="M6" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="N6" t="s">
         <v>192</v>
       </c>
       <c r="O6" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="P6" t="s">
         <v>192</v>
       </c>
       <c r="Q6" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R6" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S6" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T6" t="s">
         <v>192</v>
@@ -4994,36 +4972,42 @@
       <c r="W6" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A7" s="53">
-        <v>5</v>
-      </c>
-      <c r="B7" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="C7" s="53" t="s">
-        <v>185</v>
-      </c>
-      <c r="D7" s="53" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="53"/>
-      <c r="F7" s="53" t="s">
-        <v>192</v>
-      </c>
-      <c r="G7" s="54" t="s">
-        <v>193</v>
-      </c>
-      <c r="H7" s="54"/>
-      <c r="I7" s="54"/>
+      <c r="X6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I7" t="s">
+        <v>192</v>
+      </c>
       <c r="J7">
         <f>COUNTIF(E7:I7,"P")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K7">
         <f>ROUND(J7*10/4,0)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L7" t="s">
         <v>192</v>
@@ -5061,29 +5045,32 @@
       <c r="W7" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H8" t="s">
-        <v>192</v>
-      </c>
-      <c r="I8" t="s">
-        <v>192</v>
-      </c>
+      <c r="X7" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A8" s="53">
+        <v>5</v>
+      </c>
+      <c r="B8" s="53" t="s">
+        <v>184</v>
+      </c>
+      <c r="C8" s="53" t="s">
+        <v>185</v>
+      </c>
+      <c r="D8" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53" t="s">
+        <v>192</v>
+      </c>
+      <c r="G8" s="54" t="s">
+        <v>193</v>
+      </c>
+      <c r="H8" s="54"/>
+      <c r="I8" s="54"/>
       <c r="J8">
         <f>COUNTIF(E8:I8,"P")</f>
         <v>0</v>
@@ -5095,7 +5082,7 @@
       <c r="L8" t="s">
         <v>192</v>
       </c>
-      <c r="M8" s="54" t="s">
+      <c r="M8" t="s">
         <v>192</v>
       </c>
       <c r="N8" t="s">
@@ -5128,44 +5115,44 @@
       <c r="W8" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="H9" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I9" t="s">
         <v>192</v>
       </c>
       <c r="J9">
         <f>COUNTIF(E9:I9,"P")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <f>ROUND(J9*10/4,0)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L9" t="s">
         <v>192</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="54" t="s">
         <v>192</v>
       </c>
       <c r="N9" t="s">
@@ -5198,36 +5185,42 @@
       <c r="W9" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>53</v>
       </c>
+      <c r="E10" s="7" t="s">
+        <v>22</v>
+      </c>
       <c r="F10" s="7" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="H10" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="I10" t="s">
         <v>192</v>
       </c>
       <c r="J10">
         <f>COUNTIF(E10:I10,"P")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K10">
         <f>ROUND(J10*10/4,0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L10" t="s">
         <v>192</v>
@@ -5265,104 +5258,136 @@
       <c r="W10" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X10" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>186</v>
+        <v>90</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>91</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="H11" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="I11" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="J11">
         <f>COUNTIF(E11:I11,"P")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <f>ROUND(J11*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" t="s">
+        <v>192</v>
+      </c>
+      <c r="M11" t="s">
+        <v>192</v>
+      </c>
+      <c r="N11" t="s">
+        <v>192</v>
+      </c>
+      <c r="O11" t="s">
+        <v>192</v>
+      </c>
+      <c r="P11" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>192</v>
+      </c>
+      <c r="R11" t="s">
+        <v>192</v>
+      </c>
+      <c r="S11" t="s">
+        <v>192</v>
+      </c>
+      <c r="T11" t="s">
+        <v>192</v>
+      </c>
+      <c r="U11" t="s">
+        <v>192</v>
+      </c>
+      <c r="V11" t="s">
+        <v>192</v>
+      </c>
+      <c r="W11" t="s">
+        <v>192</v>
+      </c>
+      <c r="X11" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>9</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" t="s">
+        <v>22</v>
+      </c>
+      <c r="J12">
+        <f>COUNTIF(E12:I12,"P")</f>
+        <v>4</v>
+      </c>
+      <c r="K12">
+        <f>ROUND(J12*10/4,0)</f>
         <v>10</v>
       </c>
-      <c r="L11" t="s">
-        <v>22</v>
-      </c>
-      <c r="M11" t="s">
-        <v>22</v>
-      </c>
-      <c r="N11" t="s">
-        <v>22</v>
-      </c>
-      <c r="O11" t="s">
-        <v>22</v>
-      </c>
-      <c r="P11" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>22</v>
-      </c>
-      <c r="R11" t="s">
-        <v>22</v>
-      </c>
-      <c r="S11" t="s">
-        <v>22</v>
-      </c>
-      <c r="T11" t="s">
-        <v>192</v>
-      </c>
-      <c r="U11" t="s">
-        <v>192</v>
-      </c>
-      <c r="V11" t="s">
-        <v>192</v>
-      </c>
-      <c r="W11" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A12" s="1">
-        <v>32</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="F12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="L12" t="s">
+        <v>22</v>
+      </c>
+      <c r="M12" t="s">
+        <v>22</v>
+      </c>
+      <c r="N12" t="s">
+        <v>22</v>
+      </c>
+      <c r="O12" t="s">
+        <v>22</v>
+      </c>
       <c r="P12" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="Q12" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R12" t="s">
         <v>22</v>
       </c>
       <c r="S12" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="T12" t="s">
         <v>192</v>
@@ -5371,13 +5396,16 @@
         <v>192</v>
       </c>
       <c r="V12" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="W12" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X12" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>10</v>
       </c>
@@ -5446,8 +5474,11 @@
       <c r="W13" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X13" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>11</v>
       </c>
@@ -5514,57 +5545,28 @@
       <c r="W14" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X14" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>104</v>
+        <v>211</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>105</v>
+        <v>209</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H15" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J15">
-        <f>COUNTIF(E15:I15,"P")</f>
-        <v>3</v>
-      </c>
-      <c r="K15">
-        <f>ROUND(J15*10/4,0)</f>
-        <v>8</v>
-      </c>
-      <c r="L15" t="s">
-        <v>22</v>
-      </c>
-      <c r="M15" t="s">
-        <v>192</v>
-      </c>
-      <c r="N15" t="s">
-        <v>192</v>
-      </c>
-      <c r="O15" t="s">
-        <v>192</v>
-      </c>
-      <c r="P15" t="s">
-        <v>192</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="F15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
       <c r="Q15" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="R15" t="s">
         <v>192</v>
@@ -5576,16 +5578,19 @@
         <v>22</v>
       </c>
       <c r="U15" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="V15" t="s">
         <v>192</v>
       </c>
       <c r="W15" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+      <c r="X15" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>38</v>
       </c>
@@ -5616,8 +5621,11 @@
       <c r="W16" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X16" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>13</v>
       </c>
@@ -5683,8 +5691,11 @@
       <c r="W17" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X17" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>14</v>
       </c>
@@ -5750,8 +5761,11 @@
       <c r="W18" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X18" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>15</v>
       </c>
@@ -5823,8 +5837,11 @@
       <c r="W19" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>16</v>
       </c>
@@ -5893,8 +5910,11 @@
       <c r="W20" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X20" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>17</v>
       </c>
@@ -5963,8 +5983,11 @@
       <c r="W21" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X21" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>19</v>
       </c>
@@ -6030,8 +6053,11 @@
       <c r="W22" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X22" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>20</v>
       </c>
@@ -6100,8 +6126,11 @@
       <c r="W23" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X23" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>21</v>
       </c>
@@ -6167,8 +6196,11 @@
       <c r="W24" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X24" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>31</v>
       </c>
@@ -6214,8 +6246,11 @@
       <c r="W25" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X25" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>39</v>
       </c>
@@ -6246,8 +6281,11 @@
       <c r="W26" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X26" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>22</v>
       </c>
@@ -6316,8 +6354,11 @@
       <c r="W27" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X27" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>23</v>
       </c>
@@ -6383,8 +6424,11 @@
       <c r="W28" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X28" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>35</v>
       </c>
@@ -6421,8 +6465,11 @@
       <c r="W29" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X29" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>24</v>
       </c>
@@ -6488,8 +6535,11 @@
       <c r="W30" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X30" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>25</v>
       </c>
@@ -6555,95 +6605,66 @@
       <c r="W31" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X31" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
+        <v>36</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F32" s="7"/>
+      <c r="H32" s="7"/>
+      <c r="I32" s="7"/>
+      <c r="Q32" t="s">
+        <v>22</v>
+      </c>
+      <c r="R32" t="s">
+        <v>22</v>
+      </c>
+      <c r="S32" t="s">
+        <v>192</v>
+      </c>
+      <c r="T32" t="s">
+        <v>192</v>
+      </c>
+      <c r="U32" t="s">
+        <v>22</v>
+      </c>
+      <c r="V32" t="s">
+        <v>192</v>
+      </c>
+      <c r="W32" t="s">
+        <v>22</v>
+      </c>
+      <c r="X32" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
         <v>26</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F32" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="H32" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="J32">
-        <f>COUNTIF(E32:I32,"P")</f>
-        <v>0</v>
-      </c>
-      <c r="K32">
-        <f>ROUND(J32*10/4,0)</f>
-        <v>0</v>
-      </c>
-      <c r="L32" t="s">
-        <v>192</v>
-      </c>
-      <c r="M32" t="s">
-        <v>192</v>
-      </c>
-      <c r="N32" t="s">
-        <v>192</v>
-      </c>
-      <c r="O32" t="s">
-        <v>192</v>
-      </c>
-      <c r="P32" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>192</v>
-      </c>
-      <c r="R32" t="s">
-        <v>192</v>
-      </c>
-      <c r="S32" t="s">
-        <v>192</v>
-      </c>
-      <c r="T32" t="s">
-        <v>192</v>
-      </c>
-      <c r="U32" t="s">
-        <v>192</v>
-      </c>
-      <c r="V32" t="s">
-        <v>192</v>
-      </c>
-      <c r="W32" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A33" s="1">
-        <v>27</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>22</v>
-      </c>
       <c r="F33" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H33" s="7" t="s">
         <v>192</v>
@@ -6653,82 +6674,129 @@
       </c>
       <c r="J33">
         <f>COUNTIF(E33:I33,"P")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K33">
         <f>ROUND(J33*10/4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="L33" t="s">
+        <v>192</v>
+      </c>
+      <c r="M33" t="s">
+        <v>192</v>
+      </c>
+      <c r="N33" t="s">
+        <v>192</v>
+      </c>
+      <c r="O33" t="s">
+        <v>192</v>
+      </c>
+      <c r="P33" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>192</v>
+      </c>
+      <c r="R33" t="s">
+        <v>192</v>
+      </c>
+      <c r="S33" t="s">
+        <v>192</v>
+      </c>
+      <c r="T33" t="s">
+        <v>192</v>
+      </c>
+      <c r="U33" t="s">
+        <v>192</v>
+      </c>
+      <c r="V33" t="s">
+        <v>192</v>
+      </c>
+      <c r="W33" t="s">
+        <v>192</v>
+      </c>
+      <c r="X33" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
+        <v>27</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="H34" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="J34">
+        <f>COUNTIF(E34:I34,"P")</f>
+        <v>2</v>
+      </c>
+      <c r="K34">
+        <f>ROUND(J34*10/4,0)</f>
         <v>5</v>
       </c>
-      <c r="L33" t="s">
-        <v>192</v>
-      </c>
-      <c r="M33" t="s">
-        <v>192</v>
-      </c>
-      <c r="N33" t="s">
-        <v>192</v>
-      </c>
-      <c r="O33" t="s">
-        <v>192</v>
-      </c>
-      <c r="P33" t="s">
-        <v>192</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>192</v>
-      </c>
-      <c r="R33" t="s">
-        <v>192</v>
-      </c>
-      <c r="S33" t="s">
-        <v>192</v>
-      </c>
-      <c r="T33" t="s">
-        <v>192</v>
-      </c>
-      <c r="U33" t="s">
-        <v>192</v>
-      </c>
-      <c r="V33" t="s">
-        <v>192</v>
-      </c>
-      <c r="W33" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A34" s="1">
-        <v>37</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="F34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
+      <c r="L34" t="s">
+        <v>192</v>
+      </c>
+      <c r="M34" t="s">
+        <v>192</v>
+      </c>
+      <c r="N34" t="s">
+        <v>192</v>
+      </c>
+      <c r="O34" t="s">
+        <v>192</v>
+      </c>
+      <c r="P34" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>192</v>
+      </c>
+      <c r="R34" t="s">
+        <v>192</v>
+      </c>
       <c r="S34" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T34" t="s">
         <v>192</v>
       </c>
       <c r="U34" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="V34" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="W34" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="X34" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>30</v>
       </c>
@@ -6780,8 +6848,11 @@
       <c r="W35" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X35" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>29</v>
       </c>
@@ -6833,228 +6904,278 @@
       <c r="W36" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X36" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="F37" s="7"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
+      <c r="P37" t="s">
+        <v>22</v>
+      </c>
       <c r="Q37" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="R37" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="S37" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="T37" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="U37" t="s">
-        <v>22</v>
+        <v>192</v>
       </c>
       <c r="V37" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="W37" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="X37" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
+        <v>12</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="H38" s="57" t="s">
+        <v>22</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J38">
+        <f>COUNTIF(E38:I38,"P")</f>
+        <v>3</v>
+      </c>
+      <c r="K38">
+        <f>ROUND(J38*10/4,0)</f>
+        <v>8</v>
+      </c>
+      <c r="L38" t="s">
+        <v>22</v>
+      </c>
+      <c r="M38" t="s">
+        <v>192</v>
+      </c>
+      <c r="N38" t="s">
+        <v>192</v>
+      </c>
+      <c r="O38" t="s">
+        <v>192</v>
+      </c>
+      <c r="P38" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>192</v>
+      </c>
+      <c r="R38" t="s">
+        <v>192</v>
+      </c>
+      <c r="S38" t="s">
+        <v>22</v>
+      </c>
+      <c r="T38" t="s">
+        <v>22</v>
+      </c>
+      <c r="U38" t="s">
+        <v>192</v>
+      </c>
+      <c r="V38" t="s">
+        <v>192</v>
+      </c>
+      <c r="W38" t="s">
+        <v>192</v>
+      </c>
+      <c r="X38" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
         <v>32</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C39" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D39" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="F38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="O38" t="s">
-        <v>22</v>
-      </c>
-      <c r="P38" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>192</v>
-      </c>
-      <c r="R38" t="s">
-        <v>22</v>
-      </c>
-      <c r="S38" t="s">
-        <v>192</v>
-      </c>
-      <c r="T38" t="s">
-        <v>22</v>
-      </c>
-      <c r="U38" t="s">
-        <v>22</v>
-      </c>
-      <c r="V38" t="s">
-        <v>22</v>
-      </c>
-      <c r="W38" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A39" s="1">
+      <c r="F39" s="7"/>
+      <c r="H39" s="7"/>
+      <c r="I39" s="7"/>
+      <c r="O39" t="s">
+        <v>22</v>
+      </c>
+      <c r="P39" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>192</v>
+      </c>
+      <c r="R39" t="s">
+        <v>22</v>
+      </c>
+      <c r="S39" t="s">
+        <v>192</v>
+      </c>
+      <c r="T39" t="s">
+        <v>22</v>
+      </c>
+      <c r="U39" t="s">
+        <v>22</v>
+      </c>
+      <c r="V39" t="s">
+        <v>22</v>
+      </c>
+      <c r="W39" t="s">
+        <v>22</v>
+      </c>
+      <c r="X39" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
         <v>18</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E39" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="J39">
-        <f>COUNTIF(E39:I39,"P")</f>
+      <c r="E40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="J40">
+        <f>COUNTIF(E40:I40,"P")</f>
         <v>4</v>
       </c>
-      <c r="K39">
-        <f>ROUND(J39*10/4,0)</f>
+      <c r="K40">
+        <f>ROUND(J40*10/4,0)</f>
         <v>10</v>
       </c>
-      <c r="L39" t="s">
-        <v>22</v>
-      </c>
-      <c r="M39" t="s">
-        <v>22</v>
-      </c>
-      <c r="N39" t="s">
-        <v>22</v>
-      </c>
-      <c r="O39" t="s">
-        <v>22</v>
-      </c>
-      <c r="P39" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q39" t="s">
-        <v>22</v>
-      </c>
-      <c r="R39" t="s">
-        <v>22</v>
-      </c>
-      <c r="S39" t="s">
-        <v>22</v>
-      </c>
-      <c r="T39" t="s">
-        <v>22</v>
-      </c>
-      <c r="U39" t="s">
-        <v>22</v>
-      </c>
-      <c r="V39" t="s">
-        <v>22</v>
-      </c>
-      <c r="W39" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A40" s="1">
+      <c r="L40" t="s">
+        <v>22</v>
+      </c>
+      <c r="M40" t="s">
+        <v>22</v>
+      </c>
+      <c r="N40" t="s">
+        <v>22</v>
+      </c>
+      <c r="O40" t="s">
+        <v>22</v>
+      </c>
+      <c r="P40" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>22</v>
+      </c>
+      <c r="R40" t="s">
+        <v>22</v>
+      </c>
+      <c r="S40" t="s">
+        <v>22</v>
+      </c>
+      <c r="T40" t="s">
+        <v>22</v>
+      </c>
+      <c r="U40" t="s">
+        <v>22</v>
+      </c>
+      <c r="V40" t="s">
+        <v>22</v>
+      </c>
+      <c r="W40" t="s">
+        <v>22</v>
+      </c>
+      <c r="X40" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
         <v>28</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B41" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="D40" s="1" t="s">
+      <c r="D41" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="F40" s="7"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
-      <c r="L40" t="s">
-        <v>22</v>
-      </c>
-      <c r="M40" t="s">
-        <v>22</v>
-      </c>
-      <c r="N40" t="s">
-        <v>22</v>
-      </c>
-      <c r="O40" t="s">
-        <v>22</v>
-      </c>
-      <c r="P40" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q40" t="s">
-        <v>22</v>
-      </c>
-      <c r="R40" t="s">
-        <v>22</v>
-      </c>
-      <c r="S40" t="s">
-        <v>192</v>
-      </c>
-      <c r="T40" t="s">
-        <v>22</v>
-      </c>
-      <c r="U40" t="s">
-        <v>22</v>
-      </c>
-      <c r="V40" t="s">
-        <v>22</v>
-      </c>
-      <c r="W40" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A41" s="1">
-        <v>36</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>210</v>
       </c>
       <c r="F41" s="7"/>
       <c r="H41" s="7"/>
       <c r="I41" s="7"/>
+      <c r="L41" t="s">
+        <v>22</v>
+      </c>
+      <c r="M41" t="s">
+        <v>22</v>
+      </c>
+      <c r="N41" t="s">
+        <v>22</v>
+      </c>
+      <c r="O41" t="s">
+        <v>22</v>
+      </c>
+      <c r="P41" t="s">
+        <v>22</v>
+      </c>
       <c r="Q41" t="s">
         <v>22</v>
       </c>
@@ -7065,19 +7186,22 @@
         <v>192</v>
       </c>
       <c r="T41" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="U41" t="s">
         <v>22</v>
       </c>
       <c r="V41" t="s">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="W41" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X41" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -7086,7 +7210,7 @@
       <c r="H42" s="7"/>
       <c r="I42" s="7"/>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -7096,13 +7220,13 @@
       <c r="I43" s="7"/>
       <c r="V43" s="56"/>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:24" x14ac:dyDescent="0.2">
       <c r="D44" s="1" t="s">
         <v>191</v>
       </c>
       <c r="E44" s="1">
         <f>COUNTIF(E2:E28,"P")</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F44" s="1">
         <f>COUNTIF(F2:F28,"P")</f>
@@ -7110,15 +7234,15 @@
       </c>
       <c r="H44" s="1">
         <f>COUNTIF(H2:H28,"P")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I44" s="57">
         <f>COUNTIF(I2:I28,"P")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L44" s="1">
         <f>COUNTIF(L2:L31,"P")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M44" s="1">
         <f>COUNTIF(M2:M31,"P")</f>
@@ -7134,11 +7258,11 @@
       </c>
       <c r="P44" s="1">
         <f>COUNTIF(P2:P38,"P")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q44" s="1">
         <f>COUNTIF(Q2:Q38,"P")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R44" s="1">
         <f>COUNTIF(R2:R38,"P")</f>
@@ -7164,10 +7288,14 @@
         <f>COUNTIF(W2:W41,"P")</f>
         <v>8</v>
       </c>
+      <c r="X44" s="1">
+        <f>COUNTIF(X2:X41,"P")</f>
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:W41">
-    <sortCondition ref="W2:W41"/>
+  <sortState ref="A2:X41">
+    <sortCondition ref="X2:X41"/>
     <sortCondition ref="B2:B41"/>
   </sortState>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.0249999999999999" bottom="1.0249999999999999" header="0.78749999999999998" footer="0.78749999999999998"/>

</xml_diff>